<commit_message>
chore: refresh prices 2026-06-24 05:03 UTC
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -4,6 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Portfolio" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="MB" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="229">
   <si>
     <t>Symbol</t>
   </si>
@@ -800,7 +801,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -885,6 +886,12 @@
     <xf borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -894,6 +901,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -6527,4 +6538,313 @@
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="28" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="s">
+        <v>183</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="s">
+        <v>181</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="29" t="s">
+        <v>224</v>
+      </c>
+      <c r="B9" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="s">
+        <v>155</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="B11" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="B12" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="s">
+        <v>190</v>
+      </c>
+      <c r="B13" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="B15" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="B17" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="B18" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="29" t="s">
+        <v>207</v>
+      </c>
+      <c r="B19" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="B21" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="29" t="s">
+        <v>211</v>
+      </c>
+      <c r="B22" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="29" t="s">
+        <v>93</v>
+      </c>
+      <c r="B23" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="s">
+        <v>177</v>
+      </c>
+      <c r="B24" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C24" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="29" t="s">
+        <v>194</v>
+      </c>
+      <c r="B25" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="B26" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="C26" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: refresh prices 2026-07-07 04:14 UTC
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -1190,16 +1190,16 @@
         <v>51.86</v>
       </c>
       <c r="F2" s="7">
-        <v>96.59</v>
+        <v>96.9</v>
       </c>
       <c r="G2" s="7">
-        <v>96.59</v>
+        <v>96.9</v>
       </c>
       <c r="H2" s="7">
-        <v>44.73</v>
+        <v>45.04</v>
       </c>
       <c r="I2" s="8">
-        <v>0.8624</v>
+        <v>0.8684</v>
       </c>
       <c r="J2" s="9" t="s">
         <v>15</v>
@@ -1442,16 +1442,16 @@
         <v>110.1</v>
       </c>
       <c r="F8" s="11">
-        <v>526.5</v>
+        <v>527.0</v>
       </c>
       <c r="G8" s="11">
-        <v>526.5</v>
+        <v>527.0</v>
       </c>
       <c r="H8" s="11">
-        <v>416.4</v>
+        <v>416.9</v>
       </c>
       <c r="I8" s="12">
-        <v>3.782</v>
+        <v>3.7866</v>
       </c>
       <c r="J8" s="13" t="s">
         <v>26</v>
@@ -1484,16 +1484,16 @@
         <v>29095.0</v>
       </c>
       <c r="F9" s="11">
-        <v>807.5</v>
+        <v>807.65</v>
       </c>
       <c r="G9" s="11">
-        <v>80750.0</v>
+        <v>80765.0</v>
       </c>
       <c r="H9" s="11">
-        <v>51655.0</v>
+        <v>51670.0</v>
       </c>
       <c r="I9" s="12">
-        <v>1.7754</v>
+        <v>1.7759</v>
       </c>
       <c r="J9" s="9" t="s">
         <v>26</v>
@@ -1526,16 +1526,16 @@
         <v>59793.8</v>
       </c>
       <c r="F10" s="11">
-        <v>654.3</v>
+        <v>652.6</v>
       </c>
       <c r="G10" s="7">
-        <v>136094.4</v>
+        <v>135740.8</v>
       </c>
       <c r="H10" s="11">
-        <v>76300.6</v>
+        <v>75947.0</v>
       </c>
       <c r="I10" s="12">
-        <v>1.2761</v>
+        <v>1.2701</v>
       </c>
       <c r="J10" s="13" t="s">
         <v>15</v>
@@ -1568,16 +1568,16 @@
         <v>3887.0</v>
       </c>
       <c r="F11" s="11">
-        <v>104.0</v>
+        <v>103.9</v>
       </c>
       <c r="G11" s="11">
-        <v>16640.0</v>
+        <v>16624.0</v>
       </c>
       <c r="H11" s="11">
-        <v>12753.0</v>
+        <v>12737.0</v>
       </c>
       <c r="I11" s="14">
-        <v>3.2809</v>
+        <v>3.2768</v>
       </c>
       <c r="J11" s="15" t="s">
         <v>15</v>
@@ -1610,16 +1610,16 @@
         <v>222.45</v>
       </c>
       <c r="F12" s="11">
-        <v>385.8</v>
+        <v>386.55</v>
       </c>
       <c r="G12" s="7">
-        <v>385.8</v>
+        <v>386.55</v>
       </c>
       <c r="H12" s="11">
-        <v>163.35</v>
+        <v>164.1</v>
       </c>
       <c r="I12" s="12">
-        <v>0.7343</v>
+        <v>0.7377</v>
       </c>
       <c r="J12" s="9" t="s">
         <v>26</v>
@@ -1652,16 +1652,16 @@
         <v>588.9</v>
       </c>
       <c r="F13" s="11">
-        <v>787.45</v>
+        <v>784.1</v>
       </c>
       <c r="G13" s="7">
-        <v>787.45</v>
+        <v>784.1</v>
       </c>
       <c r="H13" s="11">
-        <v>198.55</v>
+        <v>195.2</v>
       </c>
       <c r="I13" s="14">
-        <v>0.3372</v>
+        <v>0.3315</v>
       </c>
       <c r="J13" s="15" t="s">
         <v>15</v>
@@ -1862,16 +1862,16 @@
         <v>102284.55</v>
       </c>
       <c r="F18" s="11">
-        <v>1999.1</v>
+        <v>2000.5</v>
       </c>
       <c r="G18" s="11">
-        <v>403818.2</v>
+        <v>404101.0</v>
       </c>
       <c r="H18" s="11">
-        <v>301533.65</v>
+        <v>301816.45</v>
       </c>
       <c r="I18" s="14">
-        <v>2.948</v>
+        <v>2.9508</v>
       </c>
       <c r="J18" s="15" t="s">
         <v>15</v>
@@ -1904,16 +1904,16 @@
         <v>25.25</v>
       </c>
       <c r="F19" s="11">
-        <v>138.15</v>
+        <v>138.27</v>
       </c>
       <c r="G19" s="7">
-        <v>138.15</v>
+        <v>138.27</v>
       </c>
       <c r="H19" s="11">
-        <v>112.9</v>
+        <v>113.02</v>
       </c>
       <c r="I19" s="14">
-        <v>4.4713</v>
+        <v>4.476</v>
       </c>
       <c r="J19" s="16" t="s">
         <v>15</v>
@@ -2072,16 +2072,16 @@
         <v>189012.0</v>
       </c>
       <c r="F23" s="11">
-        <v>14500.0</v>
+        <v>14524.4</v>
       </c>
       <c r="G23" s="7">
-        <v>449500.0</v>
+        <v>450256.4</v>
       </c>
       <c r="H23" s="11">
-        <v>260488.0</v>
+        <v>261244.4</v>
       </c>
       <c r="I23" s="12">
-        <v>1.3782</v>
+        <v>1.3822</v>
       </c>
       <c r="J23" s="9" t="s">
         <v>15</v>
@@ -2114,16 +2114,16 @@
         <v>11538.0</v>
       </c>
       <c r="F24" s="11">
-        <v>1394.9</v>
+        <v>1391.5</v>
       </c>
       <c r="G24" s="7">
-        <v>55796.0</v>
+        <v>55660.0</v>
       </c>
       <c r="H24" s="11">
-        <v>44258.0</v>
+        <v>44122.0</v>
       </c>
       <c r="I24" s="12">
-        <v>3.8358</v>
+        <v>3.8241</v>
       </c>
       <c r="J24" s="9" t="s">
         <v>15</v>
@@ -2156,16 +2156,16 @@
         <v>3464.5</v>
       </c>
       <c r="F25" s="7">
-        <v>1892.0</v>
+        <v>1892.45</v>
       </c>
       <c r="G25" s="7">
-        <v>5676.0</v>
+        <v>5677.35</v>
       </c>
       <c r="H25" s="7">
-        <v>2211.5</v>
+        <v>2212.85</v>
       </c>
       <c r="I25" s="17">
-        <v>0.6383</v>
+        <v>0.6387</v>
       </c>
       <c r="J25" s="16" t="s">
         <v>15</v>
@@ -2198,16 +2198,16 @@
         <v>53.6</v>
       </c>
       <c r="F26" s="7">
-        <v>514.3</v>
+        <v>514.55</v>
       </c>
       <c r="G26" s="7">
-        <v>514.3</v>
+        <v>514.55</v>
       </c>
       <c r="H26" s="7">
-        <v>460.7</v>
+        <v>460.95</v>
       </c>
       <c r="I26" s="17">
-        <v>8.5951</v>
+        <v>8.5998</v>
       </c>
       <c r="J26" s="16" t="s">
         <v>15</v>
@@ -2240,16 +2240,16 @@
         <v>415.9</v>
       </c>
       <c r="F27" s="11">
-        <v>1915.5</v>
+        <v>1915.7</v>
       </c>
       <c r="G27" s="11">
-        <v>1915.5</v>
+        <v>1915.7</v>
       </c>
       <c r="H27" s="11">
-        <v>1499.6</v>
+        <v>1499.8</v>
       </c>
       <c r="I27" s="14">
-        <v>3.6057</v>
+        <v>3.6062</v>
       </c>
       <c r="J27" s="16" t="s">
         <v>15</v>
@@ -2576,16 +2576,16 @@
         <v>24773.85</v>
       </c>
       <c r="F35" s="11">
-        <v>424.3</v>
+        <v>424.65</v>
       </c>
       <c r="G35" s="11">
-        <v>27155.2</v>
+        <v>27177.6</v>
       </c>
       <c r="H35" s="11">
-        <v>2381.35</v>
+        <v>2403.75</v>
       </c>
       <c r="I35" s="12">
-        <v>0.0961</v>
+        <v>0.097</v>
       </c>
       <c r="J35" s="9" t="s">
         <v>26</v>
@@ -2702,16 +2702,16 @@
         <v>19998.4</v>
       </c>
       <c r="F38" s="11">
-        <v>1148.0</v>
+        <v>1145.55</v>
       </c>
       <c r="G38" s="7">
-        <v>18368.0</v>
+        <v>18328.8</v>
       </c>
       <c r="H38" s="11">
-        <v>-1630.4</v>
+        <v>-1669.6</v>
       </c>
       <c r="I38" s="14">
-        <v>-0.0815</v>
+        <v>-0.0835</v>
       </c>
       <c r="J38" s="15" t="s">
         <v>26</v>
@@ -2744,16 +2744,16 @@
         <v>19800.0</v>
       </c>
       <c r="F39" s="11">
-        <v>1262.2</v>
+        <v>1262.55</v>
       </c>
       <c r="G39" s="7">
-        <v>18933.0</v>
+        <v>18938.25</v>
       </c>
       <c r="H39" s="11">
-        <v>-867.0</v>
+        <v>-861.75</v>
       </c>
       <c r="I39" s="12">
-        <v>-0.0438</v>
+        <v>-0.0435</v>
       </c>
       <c r="J39" s="9" t="s">
         <v>26</v>
@@ -2996,16 +2996,16 @@
         <v>394.05</v>
       </c>
       <c r="F45" s="11">
-        <v>334.7</v>
+        <v>334.4</v>
       </c>
       <c r="G45" s="11">
-        <v>334.7</v>
+        <v>334.4</v>
       </c>
       <c r="H45" s="11">
-        <v>-59.35</v>
+        <v>-59.65</v>
       </c>
       <c r="I45" s="12">
-        <v>-0.1506</v>
+        <v>-0.1514</v>
       </c>
       <c r="J45" s="9" t="s">
         <v>15</v>
@@ -3080,16 +3080,16 @@
         <v>11729.0</v>
       </c>
       <c r="F47" s="11">
-        <v>591.95</v>
+        <v>592.2</v>
       </c>
       <c r="G47" s="11">
-        <v>11839.0</v>
+        <v>11844.0</v>
       </c>
       <c r="H47" s="11">
-        <v>110.0</v>
+        <v>115.0</v>
       </c>
       <c r="I47" s="12">
-        <v>0.0094</v>
+        <v>0.0098</v>
       </c>
       <c r="J47" s="9" t="s">
         <v>26</v>
@@ -3122,16 +3122,16 @@
         <v>75624.0</v>
       </c>
       <c r="F48" s="11">
-        <v>3419.25</v>
+        <v>3420.3</v>
       </c>
       <c r="G48" s="7">
-        <v>68385.0</v>
+        <v>68406.0</v>
       </c>
       <c r="H48" s="11">
-        <v>-7239.0</v>
+        <v>-7218.0</v>
       </c>
       <c r="I48" s="12">
-        <v>-0.0957</v>
+        <v>-0.0954</v>
       </c>
       <c r="J48" s="13" t="s">
         <v>26</v>
@@ -3206,16 +3206,16 @@
         <v>12555.0</v>
       </c>
       <c r="F50" s="11">
-        <v>2574.0</v>
+        <v>2537.0</v>
       </c>
       <c r="G50" s="7">
-        <v>23166.0</v>
+        <v>22833.0</v>
       </c>
       <c r="H50" s="11">
-        <v>10611.0</v>
+        <v>10278.0</v>
       </c>
       <c r="I50" s="14">
-        <v>0.8452</v>
+        <v>0.8186</v>
       </c>
       <c r="J50" s="15" t="s">
         <v>26</v>
@@ -3374,16 +3374,16 @@
         <v>13793.3</v>
       </c>
       <c r="F54" s="7">
-        <v>620.5</v>
+        <v>620.75</v>
       </c>
       <c r="G54" s="7">
-        <v>14271.5</v>
+        <v>14277.25</v>
       </c>
       <c r="H54" s="7">
-        <v>478.2</v>
+        <v>483.95</v>
       </c>
       <c r="I54" s="8">
-        <v>0.0347</v>
+        <v>0.0351</v>
       </c>
       <c r="J54" s="9" t="s">
         <v>26</v>
@@ -3458,16 +3458,16 @@
         <v>45490.4</v>
       </c>
       <c r="F56" s="11">
-        <v>2083.1</v>
+        <v>2087.8</v>
       </c>
       <c r="G56" s="11">
-        <v>45828.2</v>
+        <v>45931.6</v>
       </c>
       <c r="H56" s="11">
-        <v>337.8</v>
+        <v>441.2</v>
       </c>
       <c r="I56" s="12">
-        <v>0.0074</v>
+        <v>0.0097</v>
       </c>
       <c r="J56" s="9" t="s">
         <v>26</v>
@@ -3668,16 +3668,16 @@
         <v>11919.9</v>
       </c>
       <c r="F61" s="11">
-        <v>4475.0</v>
+        <v>4453.8</v>
       </c>
       <c r="G61" s="7">
-        <v>13425.0</v>
+        <v>13361.4</v>
       </c>
       <c r="H61" s="11">
-        <v>1505.1</v>
+        <v>1441.5</v>
       </c>
       <c r="I61" s="8">
-        <v>0.1263</v>
+        <v>0.1209</v>
       </c>
       <c r="J61" s="9" t="s">
         <v>26</v>
@@ -3710,16 +3710,16 @@
         <v>72170.8</v>
       </c>
       <c r="F62" s="11">
-        <v>1872.05</v>
+        <v>1872.7</v>
       </c>
       <c r="G62" s="7">
-        <v>99218.65</v>
+        <v>99253.1</v>
       </c>
       <c r="H62" s="11">
-        <v>27047.85</v>
+        <v>27082.3</v>
       </c>
       <c r="I62" s="14">
-        <v>0.3748</v>
+        <v>0.3753</v>
       </c>
       <c r="J62" s="15" t="s">
         <v>26</v>
@@ -3794,16 +3794,16 @@
         <v>29686.25</v>
       </c>
       <c r="F64" s="11">
-        <v>796.0</v>
+        <v>800.8</v>
       </c>
       <c r="G64" s="11">
-        <v>35820.0</v>
+        <v>36036.0</v>
       </c>
       <c r="H64" s="11">
-        <v>6133.75</v>
+        <v>6349.75</v>
       </c>
       <c r="I64" s="12">
-        <v>0.2066</v>
+        <v>0.2139</v>
       </c>
       <c r="J64" s="9" t="s">
         <v>26</v>
@@ -4046,16 +4046,16 @@
         <v>10095.6</v>
       </c>
       <c r="F70" s="11">
-        <v>942.8</v>
+        <v>947.05</v>
       </c>
       <c r="G70" s="7">
-        <v>5656.8</v>
+        <v>5682.3</v>
       </c>
       <c r="H70" s="11">
-        <v>-4438.8</v>
+        <v>-4413.3</v>
       </c>
       <c r="I70" s="12">
-        <v>-0.4397</v>
+        <v>-0.4372</v>
       </c>
       <c r="J70" s="9" t="s">
         <v>26</v>
@@ -4172,16 +4172,16 @@
         <v>29813.65</v>
       </c>
       <c r="F73" s="11">
-        <v>673.0</v>
+        <v>675.9</v>
       </c>
       <c r="G73" s="7">
-        <v>26920.0</v>
+        <v>27036.0</v>
       </c>
       <c r="H73" s="11">
-        <v>-2893.65</v>
+        <v>-2777.65</v>
       </c>
       <c r="I73" s="12">
-        <v>-0.0971</v>
+        <v>-0.0932</v>
       </c>
       <c r="J73" s="9" t="s">
         <v>26</v>
@@ -4298,16 +4298,16 @@
         <v>39831.43</v>
       </c>
       <c r="F76" s="7">
-        <v>287.8</v>
+        <v>288.6</v>
       </c>
       <c r="G76" s="7">
-        <v>76842.6</v>
+        <v>77056.2</v>
       </c>
       <c r="H76" s="7">
-        <v>37011.17</v>
+        <v>37224.77</v>
       </c>
       <c r="I76" s="8">
-        <v>0.9292</v>
+        <v>0.9346</v>
       </c>
       <c r="J76" s="13" t="s">
         <v>26</v>
@@ -4676,16 +4676,16 @@
         <v>21722.1</v>
       </c>
       <c r="F85" s="11">
-        <v>1362.2</v>
+        <v>1362.85</v>
       </c>
       <c r="G85" s="7">
-        <v>42228.2</v>
+        <v>42248.35</v>
       </c>
       <c r="H85" s="11">
-        <v>20506.1</v>
+        <v>20526.25</v>
       </c>
       <c r="I85" s="12">
-        <v>0.944</v>
+        <v>0.9449</v>
       </c>
       <c r="J85" s="9" t="s">
         <v>26</v>
@@ -4844,16 +4844,16 @@
         <v>10241.0</v>
       </c>
       <c r="F89" s="11">
-        <v>151.0</v>
+        <v>151.32</v>
       </c>
       <c r="G89" s="7">
-        <v>9060.0</v>
+        <v>9079.2</v>
       </c>
       <c r="H89" s="11">
-        <v>-1181.0</v>
+        <v>-1161.8</v>
       </c>
       <c r="I89" s="17">
-        <v>-0.1153</v>
+        <v>-0.1134</v>
       </c>
       <c r="J89" s="15" t="s">
         <v>26</v>
@@ -5096,16 +5096,16 @@
         <v>68420.95</v>
       </c>
       <c r="F95" s="11">
-        <v>667.5</v>
+        <v>667.55</v>
       </c>
       <c r="G95" s="7">
-        <v>89445.0</v>
+        <v>89451.7</v>
       </c>
       <c r="H95" s="11">
-        <v>21024.05</v>
+        <v>21030.75</v>
       </c>
       <c r="I95" s="12">
-        <v>0.3073</v>
+        <v>0.3074</v>
       </c>
       <c r="J95" s="9" t="s">
         <v>26</v>
@@ -5222,16 +5222,16 @@
         <v>38589.0</v>
       </c>
       <c r="F98" s="11">
-        <v>4733.85</v>
+        <v>4736.5</v>
       </c>
       <c r="G98" s="7">
-        <v>37870.8</v>
+        <v>37892.0</v>
       </c>
       <c r="H98" s="11">
-        <v>-718.2</v>
+        <v>-697.0</v>
       </c>
       <c r="I98" s="14">
-        <v>-0.0186</v>
+        <v>-0.0181</v>
       </c>
       <c r="J98" s="15" t="s">
         <v>26</v>
@@ -5390,16 +5390,16 @@
         <v>9927.45</v>
       </c>
       <c r="F102" s="11">
-        <v>133.45</v>
+        <v>133.82</v>
       </c>
       <c r="G102" s="7">
-        <v>8674.25</v>
+        <v>8698.3</v>
       </c>
       <c r="H102" s="11">
-        <v>-1253.2</v>
+        <v>-1229.15</v>
       </c>
       <c r="I102" s="12">
-        <v>-0.1262</v>
+        <v>-0.1238</v>
       </c>
       <c r="J102" s="9" t="s">
         <v>26</v>
@@ -5642,16 +5642,16 @@
         <v>7303.1</v>
       </c>
       <c r="F108" s="11">
-        <v>1148.0</v>
+        <v>1145.55</v>
       </c>
       <c r="G108" s="11">
-        <v>8036.0</v>
+        <v>8018.85</v>
       </c>
       <c r="H108" s="11">
-        <v>732.9</v>
+        <v>715.75</v>
       </c>
       <c r="I108" s="12">
-        <v>0.1004</v>
+        <v>0.098</v>
       </c>
       <c r="J108" s="9" t="s">
         <v>26</v>
@@ -5684,16 +5684,16 @@
         <v>12681.65</v>
       </c>
       <c r="F109" s="11">
-        <v>591.95</v>
+        <v>592.2</v>
       </c>
       <c r="G109" s="11">
-        <v>13022.9</v>
+        <v>13028.4</v>
       </c>
       <c r="H109" s="11">
-        <v>341.25</v>
+        <v>346.75</v>
       </c>
       <c r="I109" s="12">
-        <v>0.0269</v>
+        <v>0.0273</v>
       </c>
       <c r="J109" s="9" t="s">
         <v>26</v>
@@ -5726,16 +5726,16 @@
         <v>11775.0</v>
       </c>
       <c r="F110" s="11">
-        <v>3419.25</v>
+        <v>3420.3</v>
       </c>
       <c r="G110" s="7">
-        <v>10257.75</v>
+        <v>10260.9</v>
       </c>
       <c r="H110" s="11">
-        <v>-1517.25</v>
+        <v>-1514.1</v>
       </c>
       <c r="I110" s="12">
-        <v>-0.1289</v>
+        <v>-0.1286</v>
       </c>
       <c r="J110" s="9" t="s">
         <v>26</v>
@@ -5768,16 +5768,16 @@
         <v>9925.04</v>
       </c>
       <c r="F111" s="11">
-        <v>113.4</v>
+        <v>113.45</v>
       </c>
       <c r="G111" s="7">
-        <v>10999.8</v>
+        <v>11004.65</v>
       </c>
       <c r="H111" s="11">
-        <v>1074.76</v>
+        <v>1079.61</v>
       </c>
       <c r="I111" s="12">
-        <v>0.1083</v>
+        <v>0.1088</v>
       </c>
       <c r="J111" s="9" t="s">
         <v>26</v>
@@ -5810,16 +5810,16 @@
         <v>9529.0</v>
       </c>
       <c r="F112" s="11">
-        <v>2083.1</v>
+        <v>2087.8</v>
       </c>
       <c r="G112" s="11">
-        <v>10415.5</v>
+        <v>10439.0</v>
       </c>
       <c r="H112" s="11">
-        <v>886.5</v>
+        <v>910.0</v>
       </c>
       <c r="I112" s="12">
-        <v>0.093</v>
+        <v>0.0955</v>
       </c>
       <c r="J112" s="9" t="s">
         <v>26</v>
@@ -5852,16 +5852,16 @@
         <v>13424.7</v>
       </c>
       <c r="F113" s="11">
-        <v>4475.0</v>
+        <v>4453.8</v>
       </c>
       <c r="G113" s="11">
-        <v>13425.0</v>
+        <v>13361.4</v>
       </c>
       <c r="H113" s="11">
-        <v>0.3</v>
+        <v>-63.3</v>
       </c>
       <c r="I113" s="12">
-        <v>0.0</v>
+        <v>-0.0047</v>
       </c>
       <c r="J113" s="13" t="s">
         <v>26</v>
@@ -5936,16 +5936,16 @@
         <v>10492.0</v>
       </c>
       <c r="F115" s="11">
-        <v>550.0</v>
+        <v>548.45</v>
       </c>
       <c r="G115" s="11">
-        <v>10450.0</v>
+        <v>10420.55</v>
       </c>
       <c r="H115" s="11">
-        <v>-42.0</v>
+        <v>-71.45</v>
       </c>
       <c r="I115" s="12">
-        <v>-0.004</v>
+        <v>-0.0068</v>
       </c>
       <c r="J115" s="9" t="s">
         <v>26</v>
@@ -5978,16 +5978,16 @@
         <v>14454.3</v>
       </c>
       <c r="F116" s="11">
-        <v>4733.85</v>
+        <v>4736.5</v>
       </c>
       <c r="G116" s="11">
-        <v>14201.55</v>
+        <v>14209.5</v>
       </c>
       <c r="H116" s="11">
-        <v>-252.75</v>
+        <v>-244.8</v>
       </c>
       <c r="I116" s="12">
-        <v>-0.0175</v>
+        <v>-0.0169</v>
       </c>
       <c r="J116" s="9" t="s">
         <v>26</v>
@@ -6020,16 +6020,16 @@
         <v>9850.1</v>
       </c>
       <c r="F117" s="11">
-        <v>463.4</v>
+        <v>464.05</v>
       </c>
       <c r="G117" s="11">
-        <v>12048.4</v>
+        <v>12065.3</v>
       </c>
       <c r="H117" s="11">
-        <v>2198.3</v>
+        <v>2215.2</v>
       </c>
       <c r="I117" s="12">
-        <v>0.2232</v>
+        <v>0.2249</v>
       </c>
       <c r="J117" s="9" t="s">
         <v>26</v>
@@ -6230,16 +6230,16 @@
         <v>1053.5</v>
       </c>
       <c r="F122" s="11">
-        <v>1849.8</v>
+        <v>1850.0</v>
       </c>
       <c r="G122" s="7">
-        <v>1849.8</v>
+        <v>1850.0</v>
       </c>
       <c r="H122" s="11">
-        <v>796.3</v>
+        <v>796.5</v>
       </c>
       <c r="I122" s="17">
-        <v>0.7559</v>
+        <v>0.7561</v>
       </c>
       <c r="J122" s="16" t="s">
         <v>15</v>
@@ -6398,16 +6398,16 @@
         <v>45461.6</v>
       </c>
       <c r="F126" s="11">
-        <v>654.3</v>
+        <v>652.6</v>
       </c>
       <c r="G126" s="7">
-        <v>157686.3</v>
+        <v>157276.6</v>
       </c>
       <c r="H126" s="11">
-        <v>112224.7</v>
+        <v>111815.0</v>
       </c>
       <c r="I126" s="14">
-        <v>2.4686</v>
+        <v>2.4595</v>
       </c>
       <c r="J126" s="15" t="s">
         <v>15</v>
@@ -6566,16 +6566,16 @@
         <v>1789.9</v>
       </c>
       <c r="F130" s="11">
-        <v>942.8</v>
+        <v>947.05</v>
       </c>
       <c r="G130" s="7">
-        <v>942.8</v>
+        <v>947.05</v>
       </c>
       <c r="H130" s="11">
-        <v>-847.1</v>
+        <v>-842.85</v>
       </c>
       <c r="I130" s="12">
-        <v>-0.4733</v>
+        <v>-0.4709</v>
       </c>
       <c r="J130" s="9" t="s">
         <v>26</v>
@@ -6608,16 +6608,16 @@
         <v>262.0</v>
       </c>
       <c r="F131" s="11">
-        <v>726.85</v>
+        <v>727.3</v>
       </c>
       <c r="G131" s="7">
-        <v>726.85</v>
+        <v>727.3</v>
       </c>
       <c r="H131" s="11">
-        <v>464.85</v>
+        <v>465.3</v>
       </c>
       <c r="I131" s="12">
-        <v>1.7742</v>
+        <v>1.776</v>
       </c>
       <c r="J131" s="9" t="s">
         <v>15</v>
@@ -6734,16 +6734,16 @@
         <v>79433.35</v>
       </c>
       <c r="F134" s="11">
-        <v>1999.1</v>
+        <v>2000.5</v>
       </c>
       <c r="G134" s="7">
-        <v>331850.6</v>
+        <v>332083.0</v>
       </c>
       <c r="H134" s="11">
-        <v>252417.25</v>
+        <v>252649.65</v>
       </c>
       <c r="I134" s="12">
-        <v>3.1777</v>
+        <v>3.1806</v>
       </c>
       <c r="J134" s="9" t="s">
         <v>15</v>
@@ -6944,16 +6944,16 @@
         <v>27243.0</v>
       </c>
       <c r="F139" s="11">
-        <v>14500.0</v>
+        <v>14500.25</v>
       </c>
       <c r="G139" s="7">
-        <v>43500.0</v>
+        <v>43500.75</v>
       </c>
       <c r="H139" s="11">
-        <v>16257.0</v>
+        <v>16257.75</v>
       </c>
       <c r="I139" s="8">
-        <v>0.5967</v>
+        <v>0.5968</v>
       </c>
       <c r="J139" s="9" t="s">
         <v>15</v>
@@ -7112,16 +7112,16 @@
         <v>885.9</v>
       </c>
       <c r="F143" s="11">
-        <v>314.5</v>
+        <v>314.9</v>
       </c>
       <c r="G143" s="7">
-        <v>3459.5</v>
+        <v>3463.9</v>
       </c>
       <c r="H143" s="11">
-        <v>2573.6</v>
+        <v>2578.0</v>
       </c>
       <c r="I143" s="14">
-        <v>2.9051</v>
+        <v>2.91</v>
       </c>
       <c r="J143" s="16" t="s">
         <v>15</v>
@@ -7154,16 +7154,16 @@
         <v>30662.25</v>
       </c>
       <c r="F144" s="11">
-        <v>1394.9</v>
+        <v>1391.5</v>
       </c>
       <c r="G144" s="11">
-        <v>111592.0</v>
+        <v>111320.0</v>
       </c>
       <c r="H144" s="11">
-        <v>80929.75</v>
+        <v>80657.75</v>
       </c>
       <c r="I144" s="12">
-        <v>2.6394</v>
+        <v>2.6305</v>
       </c>
       <c r="J144" s="9" t="s">
         <v>15</v>
@@ -7448,16 +7448,16 @@
         <v>24660.0</v>
       </c>
       <c r="F151" s="11">
-        <v>1262.2</v>
+        <v>1262.55</v>
       </c>
       <c r="G151" s="7">
-        <v>22719.6</v>
+        <v>22725.9</v>
       </c>
       <c r="H151" s="11">
-        <v>-1940.4</v>
+        <v>-1934.1</v>
       </c>
       <c r="I151" s="14">
-        <v>-0.0787</v>
+        <v>-0.0784</v>
       </c>
       <c r="J151" s="16" t="s">
         <v>26</v>
@@ -7742,16 +7742,16 @@
         <v>58774.2</v>
       </c>
       <c r="F158" s="20">
-        <v>591.95</v>
+        <v>592.2</v>
       </c>
       <c r="G158" s="21">
-        <v>62746.7</v>
+        <v>62773.2</v>
       </c>
       <c r="H158" s="20">
-        <v>3972.5</v>
+        <v>3999.0</v>
       </c>
       <c r="I158" s="12">
-        <v>0.0676</v>
+        <v>0.068</v>
       </c>
       <c r="J158" s="22" t="s">
         <v>26</v>
@@ -7825,16 +7825,16 @@
         <v>57363.6</v>
       </c>
       <c r="F160" s="7">
-        <v>3419.25</v>
+        <v>3420.3</v>
       </c>
       <c r="G160" s="7">
-        <v>61546.5</v>
+        <v>61565.4</v>
       </c>
       <c r="H160" s="25">
-        <v>4182.9</v>
+        <v>4201.8</v>
       </c>
       <c r="I160" s="26">
-        <v>0.0729</v>
+        <v>0.0732</v>
       </c>
       <c r="J160" s="2" t="s">
         <v>26</v>
@@ -8071,16 +8071,16 @@
         <v>11114.0</v>
       </c>
       <c r="F166" s="7">
-        <v>620.5</v>
+        <v>620.75</v>
       </c>
       <c r="G166" s="7">
-        <v>12410.0</v>
+        <v>12415.0</v>
       </c>
       <c r="H166" s="25">
-        <v>1296.0</v>
+        <v>1301.0</v>
       </c>
       <c r="I166" s="26">
-        <v>0.1166</v>
+        <v>0.1171</v>
       </c>
       <c r="J166" s="2" t="s">
         <v>26</v>
@@ -8153,16 +8153,16 @@
         <v>17812.6</v>
       </c>
       <c r="F168" s="7">
-        <v>2083.1</v>
+        <v>2087.8</v>
       </c>
       <c r="G168" s="7">
-        <v>18747.9</v>
+        <v>18790.2</v>
       </c>
       <c r="H168" s="25">
-        <v>935.3</v>
+        <v>977.6</v>
       </c>
       <c r="I168" s="26">
-        <v>0.0525</v>
+        <v>0.0549</v>
       </c>
       <c r="J168" s="2" t="s">
         <v>26</v>
@@ -8235,16 +8235,16 @@
         <v>86098.2</v>
       </c>
       <c r="F170" s="7">
-        <v>654.3</v>
+        <v>652.6</v>
       </c>
       <c r="G170" s="7">
-        <v>104688.0</v>
+        <v>104416.0</v>
       </c>
       <c r="H170" s="25">
-        <v>18589.8</v>
+        <v>18317.8</v>
       </c>
       <c r="I170" s="26">
-        <v>0.2159</v>
+        <v>0.2128</v>
       </c>
       <c r="J170" s="2" t="s">
         <v>15</v>
@@ -8399,16 +8399,16 @@
         <v>8567.04</v>
       </c>
       <c r="F174" s="28">
-        <v>104.0</v>
+        <v>103.9</v>
       </c>
       <c r="G174" s="28">
-        <v>14352.0</v>
+        <v>14338.2</v>
       </c>
       <c r="H174" s="28">
-        <v>5784.96</v>
+        <v>5771.16</v>
       </c>
       <c r="I174" s="29">
-        <v>0.6753</v>
+        <v>0.6736</v>
       </c>
       <c r="J174" s="1" t="s">
         <v>15</v>
@@ -8481,16 +8481,16 @@
         <v>79586.6</v>
       </c>
       <c r="F176" s="28">
-        <v>4475.0</v>
+        <v>4453.8</v>
       </c>
       <c r="G176" s="28">
-        <v>80550.0</v>
+        <v>80168.4</v>
       </c>
       <c r="H176" s="28">
-        <v>963.4</v>
+        <v>581.8</v>
       </c>
       <c r="I176" s="29">
-        <v>0.0121</v>
+        <v>0.0073</v>
       </c>
       <c r="J176" s="1" t="s">
         <v>26</v>
@@ -8522,16 +8522,16 @@
         <v>35446.4</v>
       </c>
       <c r="F177" s="28">
-        <v>1872.05</v>
+        <v>1872.7</v>
       </c>
       <c r="G177" s="28">
-        <v>56161.5</v>
+        <v>56181.0</v>
       </c>
       <c r="H177" s="28">
-        <v>20715.1</v>
+        <v>20734.6</v>
       </c>
       <c r="I177" s="29">
-        <v>0.5844</v>
+        <v>0.585</v>
       </c>
       <c r="J177" s="1" t="s">
         <v>26</v>
@@ -8850,16 +8850,16 @@
         <v>639.95</v>
       </c>
       <c r="F185" s="28">
-        <v>437.9</v>
+        <v>437.45</v>
       </c>
       <c r="G185" s="28">
-        <v>437.9</v>
+        <v>437.45</v>
       </c>
       <c r="H185" s="28">
-        <v>-202.05</v>
+        <v>-202.5</v>
       </c>
       <c r="I185" s="29">
-        <v>-0.3157</v>
+        <v>-0.3164</v>
       </c>
       <c r="J185" s="1" t="s">
         <v>26</v>
@@ -9178,16 +9178,16 @@
         <v>1679.0</v>
       </c>
       <c r="F193" s="28">
-        <v>1999.1</v>
+        <v>2000.5</v>
       </c>
       <c r="G193" s="28">
-        <v>1999.1</v>
+        <v>2000.5</v>
       </c>
       <c r="H193" s="28">
-        <v>320.1</v>
+        <v>321.5</v>
       </c>
       <c r="I193" s="29">
-        <v>0.1906</v>
+        <v>0.1915</v>
       </c>
       <c r="J193" s="1" t="s">
         <v>15</v>
@@ -9260,16 +9260,16 @@
         <v>84780.2</v>
       </c>
       <c r="F195" s="28">
-        <v>287.8</v>
+        <v>288.6</v>
       </c>
       <c r="G195" s="28">
-        <v>160016.8</v>
+        <v>160461.6</v>
       </c>
       <c r="H195" s="28">
-        <v>75236.6</v>
+        <v>75681.4</v>
       </c>
       <c r="I195" s="29">
-        <v>0.8874</v>
+        <v>0.8927</v>
       </c>
       <c r="J195" s="1" t="s">
         <v>26</v>
@@ -9383,16 +9383,16 @@
         <v>37387.9</v>
       </c>
       <c r="F198" s="28">
-        <v>550.0</v>
+        <v>548.45</v>
       </c>
       <c r="G198" s="28">
-        <v>41800.0</v>
+        <v>41682.2</v>
       </c>
       <c r="H198" s="28">
-        <v>4412.1</v>
+        <v>4294.3</v>
       </c>
       <c r="I198" s="29">
-        <v>0.118</v>
+        <v>0.1149</v>
       </c>
       <c r="J198" s="1" t="s">
         <v>26</v>
@@ -9506,16 +9506,16 @@
         <v>14635.0</v>
       </c>
       <c r="F201" s="28">
-        <v>309.45</v>
+        <v>309.55</v>
       </c>
       <c r="G201" s="28">
-        <v>15472.5</v>
+        <v>15477.5</v>
       </c>
       <c r="H201" s="28">
-        <v>837.5</v>
+        <v>842.5</v>
       </c>
       <c r="I201" s="29">
-        <v>0.0572</v>
+        <v>0.0576</v>
       </c>
       <c r="J201" s="1" t="s">
         <v>26</v>
@@ -9752,16 +9752,16 @@
         <v>9643.15</v>
       </c>
       <c r="F207" s="28">
-        <v>761.15</v>
+        <v>761.95</v>
       </c>
       <c r="G207" s="28">
-        <v>9894.95</v>
+        <v>9905.35</v>
       </c>
       <c r="H207" s="28">
-        <v>251.8</v>
+        <v>262.2</v>
       </c>
       <c r="I207" s="29">
-        <v>0.0261</v>
+        <v>0.0272</v>
       </c>
       <c r="J207" s="1" t="s">
         <v>26</v>
@@ -9793,16 +9793,16 @@
         <v>9346.2</v>
       </c>
       <c r="F208" s="28">
-        <v>1362.2</v>
+        <v>1362.85</v>
       </c>
       <c r="G208" s="28">
-        <v>16346.4</v>
+        <v>16354.2</v>
       </c>
       <c r="H208" s="28">
-        <v>7000.2</v>
+        <v>7008.0</v>
       </c>
       <c r="I208" s="29">
-        <v>0.749</v>
+        <v>0.7498</v>
       </c>
       <c r="J208" s="1" t="s">
         <v>26</v>
@@ -10080,16 +10080,16 @@
         <v>137415.0</v>
       </c>
       <c r="F215" s="28">
-        <v>14515.0</v>
+        <v>14519.18</v>
       </c>
       <c r="G215" s="28">
-        <v>217725.0</v>
+        <v>217787.7</v>
       </c>
       <c r="H215" s="28">
-        <v>80310.0</v>
+        <v>80372.7</v>
       </c>
       <c r="I215" s="29">
-        <v>0.5844</v>
+        <v>0.5849</v>
       </c>
       <c r="J215" s="1" t="s">
         <v>15</v>
@@ -10162,16 +10162,16 @@
         <v>18092.0</v>
       </c>
       <c r="F217" s="28">
-        <v>14525.0</v>
+        <v>14570.28</v>
       </c>
       <c r="G217" s="28">
-        <v>29050.0</v>
+        <v>29140.56</v>
       </c>
       <c r="H217" s="28">
-        <v>10958.0</v>
+        <v>11048.56</v>
       </c>
       <c r="I217" s="29">
-        <v>0.6057</v>
+        <v>0.6107</v>
       </c>
       <c r="J217" s="1" t="s">
         <v>15</v>
@@ -10367,16 +10367,16 @@
         <v>145192.0</v>
       </c>
       <c r="F222" s="28">
-        <v>667.5</v>
+        <v>667.55</v>
       </c>
       <c r="G222" s="28">
-        <v>165540.0</v>
+        <v>165552.4</v>
       </c>
       <c r="H222" s="28">
-        <v>20348.0</v>
+        <v>20360.4</v>
       </c>
       <c r="I222" s="29">
-        <v>0.1401</v>
+        <v>0.1402</v>
       </c>
       <c r="J222" s="1" t="s">
         <v>26</v>
@@ -10531,16 +10531,16 @@
         <v>82301.55</v>
       </c>
       <c r="F226" s="28">
-        <v>1394.9</v>
+        <v>1391.5</v>
       </c>
       <c r="G226" s="28">
-        <v>235738.1</v>
+        <v>235163.5</v>
       </c>
       <c r="H226" s="28">
-        <v>153436.55</v>
+        <v>152861.95</v>
       </c>
       <c r="I226" s="29">
-        <v>1.8643</v>
+        <v>1.8573</v>
       </c>
       <c r="J226" s="1" t="s">
         <v>15</v>
@@ -10613,16 +10613,16 @@
         <v>44852.2</v>
       </c>
       <c r="F228" s="28">
-        <v>4733.85</v>
+        <v>4736.5</v>
       </c>
       <c r="G228" s="28">
-        <v>52072.35</v>
+        <v>52101.5</v>
       </c>
       <c r="H228" s="28">
-        <v>7220.15</v>
+        <v>7249.3</v>
       </c>
       <c r="I228" s="29">
-        <v>0.161</v>
+        <v>0.1616</v>
       </c>
       <c r="J228" s="1" t="s">
         <v>26</v>
@@ -10736,16 +10736,16 @@
         <v>4617.6</v>
       </c>
       <c r="F231" s="28">
-        <v>463.4</v>
+        <v>464.05</v>
       </c>
       <c r="G231" s="28">
-        <v>5560.8</v>
+        <v>5568.6</v>
       </c>
       <c r="H231" s="28">
-        <v>943.2</v>
+        <v>951.0</v>
       </c>
       <c r="I231" s="29">
-        <v>0.2043</v>
+        <v>0.206</v>
       </c>
       <c r="J231" s="1" t="s">
         <v>26</v>
@@ -10818,16 +10818,16 @@
         <v>4377.95</v>
       </c>
       <c r="F233" s="28">
-        <v>90.0</v>
+        <v>90.38</v>
       </c>
       <c r="G233" s="28">
-        <v>3510.0</v>
+        <v>3524.82</v>
       </c>
       <c r="H233" s="28">
-        <v>-867.95</v>
+        <v>-853.13</v>
       </c>
       <c r="I233" s="29">
-        <v>-0.1983</v>
+        <v>-0.1949</v>
       </c>
       <c r="J233" s="1" t="s">
         <v>26</v>
@@ -10859,16 +10859,16 @@
         <v>19967.9</v>
       </c>
       <c r="F234" s="28">
-        <v>133.45</v>
+        <v>133.82</v>
       </c>
       <c r="G234" s="28">
-        <v>21352.0</v>
+        <v>21411.2</v>
       </c>
       <c r="H234" s="28">
-        <v>1384.1</v>
+        <v>1443.3</v>
       </c>
       <c r="I234" s="29">
-        <v>0.0693</v>
+        <v>0.0723</v>
       </c>
       <c r="J234" s="1" t="s">
         <v>26</v>
@@ -10900,16 +10900,16 @@
         <v>165.85</v>
       </c>
       <c r="F235" s="28">
-        <v>289.4</v>
+        <v>289.85</v>
       </c>
       <c r="G235" s="28">
-        <v>289.4</v>
+        <v>289.85</v>
       </c>
       <c r="H235" s="28">
-        <v>123.55</v>
+        <v>124.0</v>
       </c>
       <c r="I235" s="29">
-        <v>0.745</v>
+        <v>0.7477</v>
       </c>
       <c r="J235" s="1" t="s">
         <v>15</v>
@@ -10941,16 +10941,16 @@
         <v>56060.4</v>
       </c>
       <c r="F236" s="28">
-        <v>1543.6</v>
+        <v>1546.85</v>
       </c>
       <c r="G236" s="28">
-        <v>78723.6</v>
+        <v>78889.35</v>
       </c>
       <c r="H236" s="28">
-        <v>22663.2</v>
+        <v>22828.95</v>
       </c>
       <c r="I236" s="29">
-        <v>0.4043</v>
+        <v>0.4072</v>
       </c>
       <c r="J236" s="1" t="s">
         <v>26</v>
@@ -11187,16 +11187,16 @@
         <v>49689.7</v>
       </c>
       <c r="F242" s="28">
-        <v>850.9</v>
+        <v>851.45</v>
       </c>
       <c r="G242" s="28">
-        <v>46799.5</v>
+        <v>46829.75</v>
       </c>
       <c r="H242" s="28">
-        <v>-2890.2</v>
+        <v>-2859.95</v>
       </c>
       <c r="I242" s="29">
-        <v>-0.0582</v>
+        <v>-0.0576</v>
       </c>
       <c r="J242" s="1" t="s">
         <v>26</v>
@@ -11269,16 +11269,16 @@
         <v>39906.4</v>
       </c>
       <c r="F244" s="28">
-        <v>1148.0</v>
+        <v>1145.55</v>
       </c>
       <c r="G244" s="28">
-        <v>41328.0</v>
+        <v>41239.8</v>
       </c>
       <c r="H244" s="28">
-        <v>1421.6</v>
+        <v>1333.4</v>
       </c>
       <c r="I244" s="29">
-        <v>0.0356</v>
+        <v>0.0334</v>
       </c>
       <c r="J244" s="1" t="s">
         <v>26</v>
@@ -11310,16 +11310,16 @@
         <v>19914.4</v>
       </c>
       <c r="F245" s="28">
-        <v>169.5</v>
+        <v>169.22</v>
       </c>
       <c r="G245" s="28">
-        <v>18645.0</v>
+        <v>18614.2</v>
       </c>
       <c r="H245" s="28">
-        <v>-1269.4</v>
+        <v>-1300.2</v>
       </c>
       <c r="I245" s="29">
-        <v>-0.0637</v>
+        <v>-0.0653</v>
       </c>
       <c r="J245" s="1" t="s">
         <v>26</v>
@@ -11351,16 +11351,16 @@
         <v>53805.3</v>
       </c>
       <c r="F246" s="28">
-        <v>1262.2</v>
+        <v>1262.55</v>
       </c>
       <c r="G246" s="28">
-        <v>45439.2</v>
+        <v>45451.8</v>
       </c>
       <c r="H246" s="28">
-        <v>-8366.1</v>
+        <v>-8353.5</v>
       </c>
       <c r="I246" s="29">
-        <v>-0.1555</v>
+        <v>-0.1553</v>
       </c>
       <c r="J246" s="1" t="s">
         <v>26</v>
@@ -11433,16 +11433,16 @@
         <v>39588.85</v>
       </c>
       <c r="F248" s="28">
-        <v>591.95</v>
+        <v>592.2</v>
       </c>
       <c r="G248" s="28">
-        <v>44396.25</v>
+        <v>44415.0</v>
       </c>
       <c r="H248" s="28">
-        <v>4807.4</v>
+        <v>4826.15</v>
       </c>
       <c r="I248" s="29">
-        <v>0.1214</v>
+        <v>0.1219</v>
       </c>
       <c r="J248" s="1" t="s">
         <v>26</v>
@@ -11638,16 +11638,16 @@
         <v>26314.4</v>
       </c>
       <c r="F253" s="28">
-        <v>2083.1</v>
+        <v>2087.8</v>
       </c>
       <c r="G253" s="28">
-        <v>29163.4</v>
+        <v>29229.2</v>
       </c>
       <c r="H253" s="28">
-        <v>2849.0</v>
+        <v>2914.8</v>
       </c>
       <c r="I253" s="29">
-        <v>0.1083</v>
+        <v>0.1108</v>
       </c>
       <c r="J253" s="1" t="s">
         <v>26</v>
@@ -11720,16 +11720,16 @@
         <v>39331.9</v>
       </c>
       <c r="F255" s="28">
-        <v>4475.0</v>
+        <v>4453.8</v>
       </c>
       <c r="G255" s="28">
-        <v>40275.0</v>
+        <v>40084.2</v>
       </c>
       <c r="H255" s="28">
-        <v>943.1</v>
+        <v>752.3</v>
       </c>
       <c r="I255" s="29">
-        <v>0.024</v>
+        <v>0.0191</v>
       </c>
       <c r="J255" s="1" t="s">
         <v>26</v>
@@ -11761,16 +11761,16 @@
         <v>9990.4</v>
       </c>
       <c r="F256" s="28">
-        <v>770.6</v>
+        <v>771.45</v>
       </c>
       <c r="G256" s="28">
-        <v>10788.4</v>
+        <v>10800.3</v>
       </c>
       <c r="H256" s="28">
-        <v>798.0</v>
+        <v>809.9</v>
       </c>
       <c r="I256" s="29">
-        <v>0.0799</v>
+        <v>0.0811</v>
       </c>
       <c r="J256" s="1" t="s">
         <v>26</v>
@@ -12007,16 +12007,16 @@
         <v>99474.25</v>
       </c>
       <c r="F262" s="28">
-        <v>673.0</v>
+        <v>675.9</v>
       </c>
       <c r="G262" s="28">
-        <v>110372.0</v>
+        <v>110847.6</v>
       </c>
       <c r="H262" s="28">
-        <v>10897.75</v>
+        <v>11373.35</v>
       </c>
       <c r="I262" s="29">
-        <v>0.1096</v>
+        <v>0.1143</v>
       </c>
       <c r="J262" s="1" t="s">
         <v>26</v>
@@ -12089,16 +12089,16 @@
         <v>9896.8</v>
       </c>
       <c r="F264" s="28">
-        <v>287.8</v>
+        <v>288.6</v>
       </c>
       <c r="G264" s="28">
-        <v>11512.0</v>
+        <v>11544.0</v>
       </c>
       <c r="H264" s="28">
-        <v>1615.2</v>
+        <v>1647.2</v>
       </c>
       <c r="I264" s="29">
-        <v>0.1632</v>
+        <v>0.1664</v>
       </c>
       <c r="J264" s="1" t="s">
         <v>26</v>
@@ -12294,16 +12294,16 @@
         <v>99969.41</v>
       </c>
       <c r="F269" s="28">
-        <v>71.75</v>
+        <v>71.88</v>
       </c>
       <c r="G269" s="28">
-        <v>96288.5</v>
+        <v>96462.96</v>
       </c>
       <c r="H269" s="28">
-        <v>-3680.91</v>
+        <v>-3506.45</v>
       </c>
       <c r="I269" s="29">
-        <v>-0.0368</v>
+        <v>-0.0351</v>
       </c>
       <c r="J269" s="1" t="s">
         <v>26</v>
@@ -12417,16 +12417,16 @@
         <v>58877.0</v>
       </c>
       <c r="F272" s="28">
-        <v>4733.85</v>
+        <v>4736.5</v>
       </c>
       <c r="G272" s="28">
-        <v>61540.05</v>
+        <v>61574.5</v>
       </c>
       <c r="H272" s="28">
-        <v>2663.05</v>
+        <v>2697.5</v>
       </c>
       <c r="I272" s="29">
-        <v>0.0452</v>
+        <v>0.0458</v>
       </c>
       <c r="J272" s="1" t="s">
         <v>26</v>
@@ -12745,16 +12745,16 @@
         <v>3650.0</v>
       </c>
       <c r="F280" s="28">
-        <v>380.3</v>
+        <v>381.4</v>
       </c>
       <c r="G280" s="28">
-        <v>3803.0</v>
+        <v>3814.0</v>
       </c>
       <c r="H280" s="28">
-        <v>153.0</v>
+        <v>164.0</v>
       </c>
       <c r="I280" s="29">
-        <v>0.0419</v>
+        <v>0.0449</v>
       </c>
       <c r="J280" s="1" t="s">
         <v>26</v>
@@ -12786,16 +12786,16 @@
         <v>783.6</v>
       </c>
       <c r="F281" s="28">
-        <v>424.3</v>
+        <v>424.65</v>
       </c>
       <c r="G281" s="28">
-        <v>848.6</v>
+        <v>849.3</v>
       </c>
       <c r="H281" s="28">
-        <v>65.0</v>
+        <v>65.7</v>
       </c>
       <c r="I281" s="29">
-        <v>0.083</v>
+        <v>0.0838</v>
       </c>
       <c r="J281" s="1" t="s">
         <v>26</v>
@@ -12909,16 +12909,16 @@
         <v>12694.2</v>
       </c>
       <c r="F284" s="28">
-        <v>591.95</v>
+        <v>592.2</v>
       </c>
       <c r="G284" s="28">
-        <v>13022.9</v>
+        <v>13028.4</v>
       </c>
       <c r="H284" s="28">
-        <v>328.7</v>
+        <v>334.2</v>
       </c>
       <c r="I284" s="29">
-        <v>0.0259</v>
+        <v>0.0263</v>
       </c>
       <c r="J284" s="1" t="s">
         <v>26</v>
@@ -12950,16 +12950,16 @@
         <v>11628.6</v>
       </c>
       <c r="F285" s="28">
-        <v>4475.0</v>
+        <v>4453.8</v>
       </c>
       <c r="G285" s="28">
-        <v>13425.0</v>
+        <v>13361.4</v>
       </c>
       <c r="H285" s="28">
-        <v>1796.4</v>
+        <v>1732.8</v>
       </c>
       <c r="I285" s="29">
-        <v>0.1545</v>
+        <v>0.149</v>
       </c>
       <c r="J285" s="1" t="s">
         <v>26</v>
@@ -12991,16 +12991,16 @@
         <v>5808.0</v>
       </c>
       <c r="F286" s="28">
-        <v>2861.9</v>
+        <v>2863.6</v>
       </c>
       <c r="G286" s="28">
-        <v>5723.8</v>
+        <v>5727.2</v>
       </c>
       <c r="H286" s="28">
-        <v>-84.2</v>
+        <v>-80.8</v>
       </c>
       <c r="I286" s="29">
-        <v>-0.0145</v>
+        <v>-0.0139</v>
       </c>
       <c r="J286" s="1" t="s">
         <v>26</v>
@@ -13032,16 +13032,16 @@
         <v>1877.31</v>
       </c>
       <c r="F287" s="28">
-        <v>224.8</v>
+        <v>225.35</v>
       </c>
       <c r="G287" s="28">
-        <v>2023.2</v>
+        <v>2028.15</v>
       </c>
       <c r="H287" s="28">
-        <v>145.89</v>
+        <v>150.84</v>
       </c>
       <c r="I287" s="29">
-        <v>0.0777</v>
+        <v>0.0803</v>
       </c>
       <c r="J287" s="1" t="s">
         <v>26</v>
@@ -13073,16 +13073,16 @@
         <v>7787.1</v>
       </c>
       <c r="F288" s="28">
-        <v>287.8</v>
+        <v>288.6</v>
       </c>
       <c r="G288" s="28">
-        <v>9497.4</v>
+        <v>9523.8</v>
       </c>
       <c r="H288" s="28">
-        <v>1710.3</v>
+        <v>1736.7</v>
       </c>
       <c r="I288" s="29">
-        <v>0.2196</v>
+        <v>0.223</v>
       </c>
       <c r="J288" s="1" t="s">
         <v>26</v>
@@ -13114,16 +13114,16 @@
         <v>10923.0</v>
       </c>
       <c r="F289" s="28">
-        <v>550.0</v>
+        <v>548.45</v>
       </c>
       <c r="G289" s="28">
-        <v>11000.0</v>
+        <v>10969.0</v>
       </c>
       <c r="H289" s="28">
-        <v>77.0</v>
+        <v>46.0</v>
       </c>
       <c r="I289" s="29">
-        <v>0.007</v>
+        <v>0.0042</v>
       </c>
       <c r="J289" s="1" t="s">
         <v>26</v>
@@ -13319,13 +13319,13 @@
         <v>13167.3</v>
       </c>
       <c r="F294" s="28">
-        <v>667.5</v>
+        <v>667.55</v>
       </c>
       <c r="G294" s="28">
-        <v>15352.5</v>
+        <v>15353.65</v>
       </c>
       <c r="H294" s="28">
-        <v>2185.2</v>
+        <v>2186.35</v>
       </c>
       <c r="I294" s="29">
         <v>0.166</v>
@@ -13360,16 +13360,16 @@
         <v>14733.0</v>
       </c>
       <c r="F295" s="28">
-        <v>4733.85</v>
+        <v>4736.5</v>
       </c>
       <c r="G295" s="28">
-        <v>14201.55</v>
+        <v>14209.5</v>
       </c>
       <c r="H295" s="28">
-        <v>-531.45</v>
+        <v>-523.5</v>
       </c>
       <c r="I295" s="29">
-        <v>-0.0361</v>
+        <v>-0.0355</v>
       </c>
       <c r="J295" s="1" t="s">
         <v>26</v>
@@ -13442,16 +13442,16 @@
         <v>3496.92</v>
       </c>
       <c r="F297" s="28">
-        <v>133.45</v>
+        <v>133.82</v>
       </c>
       <c r="G297" s="28">
-        <v>3202.8</v>
+        <v>3211.68</v>
       </c>
       <c r="H297" s="28">
-        <v>-294.12</v>
+        <v>-285.24</v>
       </c>
       <c r="I297" s="29">
-        <v>-0.0841</v>
+        <v>-0.0816</v>
       </c>
       <c r="J297" s="1" t="s">
         <v>26</v>
@@ -17557,24 +17557,24 @@
     </row>
     <row r="100">
       <c r="A100" s="1" t="s">
-        <v>75</v>
+        <v>149</v>
       </c>
       <c r="B100" s="30">
-        <v>9.0</v>
+        <v>5.0</v>
       </c>
       <c r="C100" s="30">
-        <v>1395.0</v>
+        <v>2134.6</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="s">
-        <v>149</v>
+        <v>75</v>
       </c>
       <c r="B101" s="30">
-        <v>5.0</v>
+        <v>9.0</v>
       </c>
       <c r="C101" s="30">
-        <v>2134.6</v>
+        <v>1395.0</v>
       </c>
     </row>
   </sheetData>
@@ -17632,7 +17632,7 @@
         <v>1.3395</v>
       </c>
       <c r="F2" s="29">
-        <v>0.0588</v>
+        <v>0.0587</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>54</v>
@@ -17649,13 +17649,13 @@
         <v>113390.12</v>
       </c>
       <c r="C3" s="28">
-        <v>135168.75</v>
+        <v>135178.88</v>
       </c>
       <c r="D3" s="28">
-        <v>21778.63</v>
+        <v>21788.75</v>
       </c>
       <c r="E3" s="29">
-        <v>0.1921</v>
+        <v>0.1922</v>
       </c>
       <c r="F3" s="29">
         <v>0.0349</v>
@@ -17675,16 +17675,16 @@
         <v>71147.76</v>
       </c>
       <c r="C4" s="28">
-        <v>128934.4</v>
+        <v>129292.8</v>
       </c>
       <c r="D4" s="28">
-        <v>57786.64</v>
+        <v>58145.04</v>
       </c>
       <c r="E4" s="29">
-        <v>0.8122</v>
+        <v>0.8172</v>
       </c>
       <c r="F4" s="29">
-        <v>0.0333</v>
+        <v>0.0334</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>33</v>
@@ -17753,13 +17753,13 @@
         <v>85752.75</v>
       </c>
       <c r="C7" s="28">
-        <v>89943.15</v>
+        <v>89993.5</v>
       </c>
       <c r="D7" s="28">
-        <v>4190.4</v>
+        <v>4240.75</v>
       </c>
       <c r="E7" s="29">
-        <v>0.0489</v>
+        <v>0.0495</v>
       </c>
       <c r="F7" s="29">
         <v>0.0232</v>
@@ -17857,16 +17857,16 @@
         <v>77945.85</v>
       </c>
       <c r="C11" s="28">
-        <v>80550.0</v>
+        <v>80168.4</v>
       </c>
       <c r="D11" s="28">
-        <v>2604.15</v>
+        <v>2222.55</v>
       </c>
       <c r="E11" s="29">
-        <v>0.0334</v>
+        <v>0.0285</v>
       </c>
       <c r="F11" s="29">
-        <v>0.0208</v>
+        <v>0.0207</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>54</v>
@@ -17883,13 +17883,13 @@
         <v>53808.6</v>
       </c>
       <c r="C12" s="28">
-        <v>77690.07</v>
+        <v>77717.05</v>
       </c>
       <c r="D12" s="28">
-        <v>23881.48</v>
+        <v>23908.45</v>
       </c>
       <c r="E12" s="29">
-        <v>0.4438</v>
+        <v>0.4443</v>
       </c>
       <c r="F12" s="29">
         <v>0.0201</v>
@@ -17961,13 +17961,13 @@
         <v>67733.95</v>
       </c>
       <c r="C15" s="28">
-        <v>72513.88</v>
+        <v>72544.5</v>
       </c>
       <c r="D15" s="28">
-        <v>4779.93</v>
+        <v>4810.55</v>
       </c>
       <c r="E15" s="29">
-        <v>0.0706</v>
+        <v>0.071</v>
       </c>
       <c r="F15" s="29">
         <v>0.0187</v>
@@ -18013,13 +18013,13 @@
         <v>72381.3</v>
       </c>
       <c r="C17" s="28">
-        <v>70094.62</v>
+        <v>70116.15</v>
       </c>
       <c r="D17" s="28">
-        <v>-2286.67</v>
+        <v>-2265.15</v>
       </c>
       <c r="E17" s="29">
-        <v>-0.0316</v>
+        <v>-0.0313</v>
       </c>
       <c r="F17" s="29">
         <v>0.0181</v>
@@ -18039,16 +18039,16 @@
         <v>64643.95</v>
       </c>
       <c r="C18" s="28">
-        <v>68646.0</v>
+        <v>68941.8</v>
       </c>
       <c r="D18" s="28">
-        <v>4002.05</v>
+        <v>4297.85</v>
       </c>
       <c r="E18" s="29">
-        <v>0.0619</v>
+        <v>0.0665</v>
       </c>
       <c r="F18" s="29">
-        <v>0.0177</v>
+        <v>0.0178</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>17</v>
@@ -18221,13 +18221,13 @@
         <v>49573.2</v>
       </c>
       <c r="C25" s="28">
-        <v>52077.5</v>
+        <v>52195.0</v>
       </c>
       <c r="D25" s="28">
-        <v>2504.3</v>
+        <v>2621.8</v>
       </c>
       <c r="E25" s="29">
-        <v>0.0505</v>
+        <v>0.0529</v>
       </c>
       <c r="F25" s="29">
         <v>0.0135</v>
@@ -18247,13 +18247,13 @@
         <v>46334.02</v>
       </c>
       <c r="C26" s="28">
-        <v>51514.2</v>
+        <v>51544.8</v>
       </c>
       <c r="D26" s="28">
-        <v>5180.18</v>
+        <v>5210.78</v>
       </c>
       <c r="E26" s="29">
-        <v>0.1118</v>
+        <v>0.1125</v>
       </c>
       <c r="F26" s="29">
         <v>0.0133</v>
@@ -18325,16 +18325,16 @@
         <v>49984.7</v>
       </c>
       <c r="C29" s="28">
-        <v>48144.25</v>
+        <v>48231.48</v>
       </c>
       <c r="D29" s="28">
-        <v>-1840.45</v>
+        <v>-1753.22</v>
       </c>
       <c r="E29" s="29">
-        <v>-0.0368</v>
+        <v>-0.0351</v>
       </c>
       <c r="F29" s="29">
-        <v>0.0124</v>
+        <v>0.0125</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>62</v>
@@ -18377,13 +18377,13 @@
         <v>49132.65</v>
       </c>
       <c r="C31" s="28">
-        <v>43545.9</v>
+        <v>43557.97</v>
       </c>
       <c r="D31" s="28">
-        <v>-5586.75</v>
+        <v>-5574.67</v>
       </c>
       <c r="E31" s="29">
-        <v>-0.1137</v>
+        <v>-0.1135</v>
       </c>
       <c r="F31" s="29">
         <v>0.0113</v>
@@ -18507,13 +18507,13 @@
         <v>14547.5</v>
       </c>
       <c r="C36" s="28">
-        <v>40375.0</v>
+        <v>40382.5</v>
       </c>
       <c r="D36" s="28">
-        <v>25827.5</v>
+        <v>25835.0</v>
       </c>
       <c r="E36" s="29">
-        <v>1.7754</v>
+        <v>1.7759</v>
       </c>
       <c r="F36" s="29">
         <v>0.0104</v>
@@ -18533,13 +18533,13 @@
         <v>28030.2</v>
       </c>
       <c r="C37" s="28">
-        <v>39361.8</v>
+        <v>39444.67</v>
       </c>
       <c r="D37" s="28">
-        <v>11331.6</v>
+        <v>11414.48</v>
       </c>
       <c r="E37" s="29">
-        <v>0.4043</v>
+        <v>0.4072</v>
       </c>
       <c r="F37" s="29">
         <v>0.0102</v>
@@ -18663,13 +18663,13 @@
         <v>21235.27</v>
       </c>
       <c r="C42" s="28">
-        <v>36915.78</v>
+        <v>36954.58</v>
       </c>
       <c r="D42" s="28">
-        <v>15680.5</v>
+        <v>15719.3</v>
       </c>
       <c r="E42" s="29">
-        <v>0.7384</v>
+        <v>0.7402</v>
       </c>
       <c r="F42" s="29">
         <v>0.0095</v>
@@ -18741,16 +18741,16 @@
         <v>33603.95</v>
       </c>
       <c r="C45" s="28">
-        <v>33866.0</v>
+        <v>33793.72</v>
       </c>
       <c r="D45" s="28">
-        <v>262.05</v>
+        <v>189.78</v>
       </c>
       <c r="E45" s="29">
-        <v>0.0078</v>
+        <v>0.0056</v>
       </c>
       <c r="F45" s="29">
-        <v>0.0088</v>
+        <v>0.0087</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>62</v>
@@ -18793,16 +18793,16 @@
         <v>29401.45</v>
       </c>
       <c r="C47" s="28">
-        <v>31625.0</v>
+        <v>31535.88</v>
       </c>
       <c r="D47" s="28">
-        <v>2223.55</v>
+        <v>2134.43</v>
       </c>
       <c r="E47" s="29">
-        <v>0.0756</v>
+        <v>0.0726</v>
       </c>
       <c r="F47" s="29">
-        <v>0.0082</v>
+        <v>0.0081</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>62</v>
@@ -18871,13 +18871,13 @@
         <v>15534.15</v>
       </c>
       <c r="C50" s="28">
-        <v>29287.3</v>
+        <v>29301.27</v>
       </c>
       <c r="D50" s="28">
-        <v>13753.15</v>
+        <v>13767.13</v>
       </c>
       <c r="E50" s="29">
-        <v>0.8853</v>
+        <v>0.8862</v>
       </c>
       <c r="F50" s="29">
         <v>0.0076</v>
@@ -18958,7 +18958,7 @@
         <v>0.1003</v>
       </c>
       <c r="F53" s="29">
-        <v>0.0072</v>
+        <v>0.0071</v>
       </c>
       <c r="G53" s="1" t="s">
         <v>17</v>
@@ -18975,13 +18975,13 @@
         <v>26249.6</v>
       </c>
       <c r="C54" s="28">
-        <v>27571.75</v>
+        <v>27651.5</v>
       </c>
       <c r="D54" s="28">
-        <v>1322.15</v>
+        <v>1401.9</v>
       </c>
       <c r="E54" s="29">
-        <v>0.0504</v>
+        <v>0.0534</v>
       </c>
       <c r="F54" s="29">
         <v>0.0071</v>
@@ -19088,7 +19088,7 @@
         <v>-0.0154</v>
       </c>
       <c r="F58" s="29">
-        <v>0.0064</v>
+        <v>0.0063</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>17</v>
@@ -19105,16 +19105,16 @@
         <v>23284.61</v>
       </c>
       <c r="C59" s="28">
-        <v>24166.0</v>
+        <v>24225.12</v>
       </c>
       <c r="D59" s="28">
-        <v>881.39</v>
+        <v>940.51</v>
       </c>
       <c r="E59" s="29">
-        <v>0.0379</v>
+        <v>0.0404</v>
       </c>
       <c r="F59" s="29">
-        <v>0.0062</v>
+        <v>0.0063</v>
       </c>
       <c r="G59" s="1" t="s">
         <v>17</v>
@@ -19131,13 +19131,13 @@
         <v>24844.85</v>
       </c>
       <c r="C60" s="28">
-        <v>23399.75</v>
+        <v>23414.88</v>
       </c>
       <c r="D60" s="28">
-        <v>-1445.1</v>
+        <v>-1429.97</v>
       </c>
       <c r="E60" s="29">
-        <v>-0.0582</v>
+        <v>-0.0576</v>
       </c>
       <c r="F60" s="29">
         <v>0.006</v>
@@ -19365,16 +19365,16 @@
         <v>14843.12</v>
       </c>
       <c r="C69" s="28">
-        <v>17910.0</v>
+        <v>18018.0</v>
       </c>
       <c r="D69" s="28">
-        <v>3066.88</v>
+        <v>3174.88</v>
       </c>
       <c r="E69" s="29">
-        <v>0.2066</v>
+        <v>0.2139</v>
       </c>
       <c r="F69" s="29">
-        <v>0.0046</v>
+        <v>0.0047</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>17</v>
@@ -19443,13 +19443,13 @@
         <v>16696.13</v>
       </c>
       <c r="C72" s="28">
-        <v>16614.52</v>
+        <v>16660.59</v>
       </c>
       <c r="D72" s="28">
-        <v>-81.61</v>
+        <v>-35.54</v>
       </c>
       <c r="E72" s="29">
-        <v>-0.0049</v>
+        <v>-0.0021</v>
       </c>
       <c r="F72" s="29">
         <v>0.0043</v>
@@ -19599,13 +19599,13 @@
         <v>12778.72</v>
       </c>
       <c r="C78" s="28">
-        <v>14001.9</v>
+        <v>14013.45</v>
       </c>
       <c r="D78" s="28">
-        <v>1223.18</v>
+        <v>1234.73</v>
       </c>
       <c r="E78" s="29">
-        <v>0.0957</v>
+        <v>0.0966</v>
       </c>
       <c r="F78" s="29">
         <v>0.0036</v>
@@ -19703,13 +19703,13 @@
         <v>12453.65</v>
       </c>
       <c r="C82" s="28">
-        <v>13340.75</v>
+        <v>13346.12</v>
       </c>
       <c r="D82" s="28">
-        <v>887.1</v>
+        <v>892.48</v>
       </c>
       <c r="E82" s="29">
-        <v>0.0712</v>
+        <v>0.0717</v>
       </c>
       <c r="F82" s="29">
         <v>0.0034</v>
@@ -19729,13 +19729,13 @@
         <v>17016.17</v>
       </c>
       <c r="C83" s="28">
-        <v>12918.05</v>
+        <v>12904.77</v>
       </c>
       <c r="D83" s="28">
-        <v>-4098.12</v>
+        <v>-4111.4</v>
       </c>
       <c r="E83" s="29">
-        <v>-0.2408</v>
+        <v>-0.2416</v>
       </c>
       <c r="F83" s="29">
         <v>0.0033</v>
@@ -19781,16 +19781,16 @@
         <v>6277.5</v>
       </c>
       <c r="C85" s="28">
-        <v>11583.0</v>
+        <v>11416.5</v>
       </c>
       <c r="D85" s="28">
-        <v>5305.5</v>
+        <v>5139.0</v>
       </c>
       <c r="E85" s="29">
-        <v>0.8452</v>
+        <v>0.8186</v>
       </c>
       <c r="F85" s="29">
-        <v>0.003</v>
+        <v>0.0029</v>
       </c>
       <c r="G85" s="1" t="s">
         <v>17</v>
@@ -19920,7 +19920,7 @@
         <v>-0.0044</v>
       </c>
       <c r="F90" s="29">
-        <v>0.0026</v>
+        <v>0.0025</v>
       </c>
       <c r="G90" s="1" t="s">
         <v>17</v>
@@ -20093,13 +20093,13 @@
         <v>9957.2</v>
       </c>
       <c r="C97" s="28">
-        <v>9322.5</v>
+        <v>9307.1</v>
       </c>
       <c r="D97" s="28">
-        <v>-634.7</v>
+        <v>-650.1</v>
       </c>
       <c r="E97" s="29">
-        <v>-0.0637</v>
+        <v>-0.0653</v>
       </c>
       <c r="F97" s="29">
         <v>0.0024</v>
@@ -20171,13 +20171,13 @@
         <v>7317.5</v>
       </c>
       <c r="C100" s="28">
-        <v>7736.25</v>
+        <v>7738.75</v>
       </c>
       <c r="D100" s="28">
-        <v>418.75</v>
+        <v>421.25</v>
       </c>
       <c r="E100" s="29">
-        <v>0.0572</v>
+        <v>0.0576</v>
       </c>
       <c r="F100" s="29">
         <v>0.002</v>
@@ -20249,13 +20249,13 @@
         <v>4995.2</v>
       </c>
       <c r="C103" s="28">
-        <v>5394.2</v>
+        <v>5400.15</v>
       </c>
       <c r="D103" s="28">
-        <v>399.0</v>
+        <v>404.95</v>
       </c>
       <c r="E103" s="29">
-        <v>0.0799</v>
+        <v>0.0811</v>
       </c>
       <c r="F103" s="29">
         <v>0.0014</v>
@@ -20353,13 +20353,13 @@
         <v>2188.98</v>
       </c>
       <c r="C107" s="28">
-        <v>1755.0</v>
+        <v>1762.41</v>
       </c>
       <c r="D107" s="28">
-        <v>-433.98</v>
+        <v>-426.57</v>
       </c>
       <c r="E107" s="29">
-        <v>-0.1983</v>
+        <v>-0.1949</v>
       </c>
       <c r="F107" s="29">
         <v>5.0E-4</v>
@@ -20405,13 +20405,13 @@
         <v>222.45</v>
       </c>
       <c r="C109" s="28">
-        <v>385.8</v>
+        <v>386.55</v>
       </c>
       <c r="D109" s="28">
-        <v>163.35</v>
+        <v>164.1</v>
       </c>
       <c r="E109" s="29">
-        <v>0.7343</v>
+        <v>0.7377</v>
       </c>
       <c r="F109" s="29">
         <v>1.0E-4</v>
@@ -20499,16 +20499,16 @@
         <v>14599.99</v>
       </c>
       <c r="F2" s="28">
-        <v>3450860.42</v>
+        <v>3451770.83</v>
       </c>
       <c r="G2" s="28">
-        <v>1507881.04</v>
+        <v>1508791.45</v>
       </c>
       <c r="H2" s="29">
-        <v>0.7761</v>
+        <v>0.7765</v>
       </c>
       <c r="I2" s="29">
-        <v>0.2051</v>
+        <v>0.2052</v>
       </c>
       <c r="J2" s="29" t="s">
         <v>23</v>
@@ -20628,19 +20628,19 @@
         <v>183396.9</v>
       </c>
       <c r="E5" s="28">
-        <v>1999.1</v>
+        <v>2000.5</v>
       </c>
       <c r="F5" s="28">
-        <v>737667.9</v>
+        <v>738184.5</v>
       </c>
       <c r="G5" s="28">
-        <v>554271.0</v>
+        <v>554787.6</v>
       </c>
       <c r="H5" s="29">
-        <v>3.0222</v>
+        <v>3.0251</v>
       </c>
       <c r="I5" s="29">
-        <v>0.0438</v>
+        <v>0.0439</v>
       </c>
       <c r="J5" s="29">
         <v>0.063</v>
@@ -20716,22 +20716,22 @@
         <v>124501.8</v>
       </c>
       <c r="E7" s="28">
-        <v>1394.9</v>
+        <v>1391.5</v>
       </c>
       <c r="F7" s="28">
-        <v>403126.1</v>
+        <v>402143.5</v>
       </c>
       <c r="G7" s="28">
-        <v>278624.3</v>
+        <v>277641.7</v>
       </c>
       <c r="H7" s="29">
-        <v>2.2379</v>
+        <v>2.23</v>
       </c>
       <c r="I7" s="29">
-        <v>0.024</v>
+        <v>0.0239</v>
       </c>
       <c r="J7" s="29">
-        <v>0.0344</v>
+        <v>0.0343</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>15</v>
@@ -20760,22 +20760,22 @@
         <v>191353.6</v>
       </c>
       <c r="E8" s="28">
-        <v>654.3</v>
+        <v>652.6</v>
       </c>
       <c r="F8" s="28">
-        <v>398468.7</v>
+        <v>397433.4</v>
       </c>
       <c r="G8" s="28">
-        <v>207115.1</v>
+        <v>206079.8</v>
       </c>
       <c r="H8" s="29">
-        <v>1.0824</v>
+        <v>1.077</v>
       </c>
       <c r="I8" s="29">
-        <v>0.0237</v>
+        <v>0.0236</v>
       </c>
       <c r="J8" s="29">
-        <v>0.034</v>
+        <v>0.0339</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>15</v>
@@ -20804,16 +20804,16 @@
         <v>226780.25</v>
       </c>
       <c r="E9" s="28">
-        <v>667.5</v>
+        <v>667.55</v>
       </c>
       <c r="F9" s="28">
-        <v>270337.5</v>
+        <v>270357.75</v>
       </c>
       <c r="G9" s="28">
-        <v>43557.25</v>
+        <v>43577.5</v>
       </c>
       <c r="H9" s="29">
-        <v>0.1921</v>
+        <v>0.1922</v>
       </c>
       <c r="I9" s="29">
         <v>0.0161</v>
@@ -20848,22 +20848,22 @@
         <v>142295.53</v>
       </c>
       <c r="E10" s="28">
-        <v>287.8</v>
+        <v>288.6</v>
       </c>
       <c r="F10" s="28">
-        <v>257868.8</v>
+        <v>258585.6</v>
       </c>
       <c r="G10" s="28">
-        <v>115573.27</v>
+        <v>116290.07</v>
       </c>
       <c r="H10" s="29">
-        <v>0.8122</v>
+        <v>0.8172</v>
       </c>
       <c r="I10" s="29">
-        <v>0.0153</v>
+        <v>0.0154</v>
       </c>
       <c r="J10" s="29">
-        <v>0.022</v>
+        <v>0.0221</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>26</v>
@@ -20980,13 +20980,13 @@
         <v>22697.7</v>
       </c>
       <c r="E13" s="28">
-        <v>1849.8</v>
+        <v>1850.0</v>
       </c>
       <c r="F13" s="28">
-        <v>186849.8</v>
+        <v>186850.0</v>
       </c>
       <c r="G13" s="28">
-        <v>164152.1</v>
+        <v>164152.3</v>
       </c>
       <c r="H13" s="29">
         <v>7.2321</v>
@@ -20995,7 +20995,7 @@
         <v>0.0111</v>
       </c>
       <c r="J13" s="29">
-        <v>0.0159</v>
+        <v>0.016</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>15</v>
@@ -21112,16 +21112,16 @@
         <v>171505.5</v>
       </c>
       <c r="E16" s="28">
-        <v>4733.85</v>
+        <v>4736.5</v>
       </c>
       <c r="F16" s="28">
-        <v>179886.3</v>
+        <v>179987.0</v>
       </c>
       <c r="G16" s="28">
-        <v>8380.8</v>
+        <v>8481.5</v>
       </c>
       <c r="H16" s="29">
-        <v>0.0489</v>
+        <v>0.0495</v>
       </c>
       <c r="I16" s="29">
         <v>0.0107</v>
@@ -21288,22 +21288,22 @@
         <v>155891.7</v>
       </c>
       <c r="E20" s="28">
-        <v>4475.0</v>
+        <v>4453.8</v>
       </c>
       <c r="F20" s="28">
-        <v>161100.0</v>
+        <v>160336.8</v>
       </c>
       <c r="G20" s="28">
-        <v>5208.3</v>
+        <v>4445.1</v>
       </c>
       <c r="H20" s="29">
-        <v>0.0334</v>
+        <v>0.0285</v>
       </c>
       <c r="I20" s="29">
-        <v>0.0096</v>
+        <v>0.0095</v>
       </c>
       <c r="J20" s="29">
-        <v>0.0138</v>
+        <v>0.0137</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>26</v>
@@ -21332,16 +21332,16 @@
         <v>107617.2</v>
       </c>
       <c r="E21" s="28">
-        <v>1872.05</v>
+        <v>1872.7</v>
       </c>
       <c r="F21" s="28">
-        <v>155380.15</v>
+        <v>155434.1</v>
       </c>
       <c r="G21" s="28">
-        <v>47762.95</v>
+        <v>47816.9</v>
       </c>
       <c r="H21" s="29">
-        <v>0.4438</v>
+        <v>0.4443</v>
       </c>
       <c r="I21" s="29">
         <v>0.0092</v>
@@ -21464,16 +21464,16 @@
         <v>135467.9</v>
       </c>
       <c r="E24" s="28">
-        <v>591.95</v>
+        <v>592.2</v>
       </c>
       <c r="F24" s="28">
-        <v>145027.75</v>
+        <v>145089.0</v>
       </c>
       <c r="G24" s="28">
-        <v>9559.85</v>
+        <v>9621.1</v>
       </c>
       <c r="H24" s="29">
-        <v>0.0706</v>
+        <v>0.071</v>
       </c>
       <c r="I24" s="29">
         <v>0.0086</v>
@@ -21596,16 +21596,16 @@
         <v>144762.6</v>
       </c>
       <c r="E27" s="28">
-        <v>3419.25</v>
+        <v>3420.3</v>
       </c>
       <c r="F27" s="28">
-        <v>140189.25</v>
+        <v>140232.3</v>
       </c>
       <c r="G27" s="28">
-        <v>-4573.35</v>
+        <v>-4530.3</v>
       </c>
       <c r="H27" s="29">
-        <v>-0.0316</v>
+        <v>-0.0313</v>
       </c>
       <c r="I27" s="29">
         <v>0.0083</v>
@@ -21640,22 +21640,22 @@
         <v>129287.9</v>
       </c>
       <c r="E28" s="28">
-        <v>673.0</v>
+        <v>675.9</v>
       </c>
       <c r="F28" s="28">
-        <v>137292.0</v>
+        <v>137883.6</v>
       </c>
       <c r="G28" s="28">
-        <v>8004.1</v>
+        <v>8595.7</v>
       </c>
       <c r="H28" s="29">
-        <v>0.0619</v>
+        <v>0.0665</v>
       </c>
       <c r="I28" s="29">
         <v>0.0082</v>
       </c>
       <c r="J28" s="29">
-        <v>0.0117</v>
+        <v>0.0118</v>
       </c>
       <c r="K28" s="1" t="s">
         <v>26</v>
@@ -22039,13 +22039,13 @@
         <v>463.4</v>
       </c>
       <c r="F37" s="28">
-        <v>113996.4</v>
+        <v>114021.1</v>
       </c>
       <c r="G37" s="28">
-        <v>19490.3</v>
+        <v>19515.0</v>
       </c>
       <c r="H37" s="29">
-        <v>0.2062</v>
+        <v>0.2065</v>
       </c>
       <c r="I37" s="29">
         <v>0.0068</v>
@@ -22124,16 +22124,16 @@
         <v>99146.4</v>
       </c>
       <c r="E39" s="28">
-        <v>2083.1</v>
+        <v>2087.8</v>
       </c>
       <c r="F39" s="28">
-        <v>104155.0</v>
+        <v>104390.0</v>
       </c>
       <c r="G39" s="28">
-        <v>5008.6</v>
+        <v>5243.6</v>
       </c>
       <c r="H39" s="29">
-        <v>0.0505</v>
+        <v>0.0529</v>
       </c>
       <c r="I39" s="29">
         <v>0.0062</v>
@@ -22168,13 +22168,13 @@
         <v>92668.05</v>
       </c>
       <c r="E40" s="28">
-        <v>2861.9</v>
+        <v>2863.6</v>
       </c>
       <c r="F40" s="28">
-        <v>103028.4</v>
+        <v>103031.8</v>
       </c>
       <c r="G40" s="28">
-        <v>10360.35</v>
+        <v>10363.75</v>
       </c>
       <c r="H40" s="29">
         <v>0.1118</v>
@@ -22432,16 +22432,16 @@
         <v>99969.41</v>
       </c>
       <c r="E46" s="28">
-        <v>71.75</v>
+        <v>71.88</v>
       </c>
       <c r="F46" s="28">
-        <v>96288.5</v>
+        <v>96462.96</v>
       </c>
       <c r="G46" s="28">
-        <v>-3680.91</v>
+        <v>-3506.45</v>
       </c>
       <c r="H46" s="29">
-        <v>-0.0368</v>
+        <v>-0.0351</v>
       </c>
       <c r="I46" s="29">
         <v>0.0057</v>
@@ -22520,16 +22520,16 @@
         <v>98265.3</v>
       </c>
       <c r="E48" s="28">
-        <v>1262.2</v>
+        <v>1262.55</v>
       </c>
       <c r="F48" s="28">
-        <v>87091.8</v>
+        <v>87115.95</v>
       </c>
       <c r="G48" s="28">
-        <v>-11173.5</v>
+        <v>-11149.35</v>
       </c>
       <c r="H48" s="29">
-        <v>-0.1137</v>
+        <v>-0.1135</v>
       </c>
       <c r="I48" s="29">
         <v>0.0052</v>
@@ -22743,13 +22743,13 @@
         <v>151.32</v>
       </c>
       <c r="F53" s="28">
-        <v>82601.52</v>
+        <v>82620.72</v>
       </c>
       <c r="G53" s="28">
-        <v>8393.25</v>
+        <v>8412.45</v>
       </c>
       <c r="H53" s="29">
-        <v>0.1131</v>
+        <v>0.1134</v>
       </c>
       <c r="I53" s="29">
         <v>0.0049</v>
@@ -22872,16 +22872,16 @@
         <v>29095.0</v>
       </c>
       <c r="E56" s="28">
-        <v>807.5</v>
+        <v>807.65</v>
       </c>
       <c r="F56" s="28">
-        <v>80750.0</v>
+        <v>80765.0</v>
       </c>
       <c r="G56" s="28">
-        <v>51655.0</v>
+        <v>51670.0</v>
       </c>
       <c r="H56" s="29">
-        <v>1.7754</v>
+        <v>1.7759</v>
       </c>
       <c r="I56" s="29">
         <v>0.0048</v>
@@ -22916,16 +22916,16 @@
         <v>56060.4</v>
       </c>
       <c r="E57" s="28">
-        <v>1543.6</v>
+        <v>1546.85</v>
       </c>
       <c r="F57" s="28">
-        <v>78723.6</v>
+        <v>78889.35</v>
       </c>
       <c r="G57" s="28">
-        <v>22663.2</v>
+        <v>22828.95</v>
       </c>
       <c r="H57" s="29">
-        <v>0.4043</v>
+        <v>0.4072</v>
       </c>
       <c r="I57" s="29">
         <v>0.0047</v>
@@ -23180,16 +23180,16 @@
         <v>42470.55</v>
       </c>
       <c r="E63" s="28">
-        <v>761.15</v>
+        <v>761.95</v>
       </c>
       <c r="F63" s="28">
-        <v>73831.55</v>
+        <v>73841.95</v>
       </c>
       <c r="G63" s="28">
-        <v>31361.0</v>
+        <v>31371.4</v>
       </c>
       <c r="H63" s="29">
-        <v>0.7384</v>
+        <v>0.7387</v>
       </c>
       <c r="I63" s="29">
         <v>0.0044</v>
@@ -23312,16 +23312,16 @@
         <v>67207.9</v>
       </c>
       <c r="E66" s="28">
-        <v>1148.0</v>
+        <v>1145.55</v>
       </c>
       <c r="F66" s="28">
-        <v>67732.0</v>
+        <v>67587.45</v>
       </c>
       <c r="G66" s="28">
-        <v>524.1</v>
+        <v>379.55</v>
       </c>
       <c r="H66" s="29">
-        <v>0.0078</v>
+        <v>0.0056</v>
       </c>
       <c r="I66" s="29">
         <v>0.004</v>
@@ -23444,19 +23444,19 @@
         <v>58802.9</v>
       </c>
       <c r="E69" s="28">
-        <v>550.0</v>
+        <v>548.45</v>
       </c>
       <c r="F69" s="28">
-        <v>63250.0</v>
+        <v>63071.75</v>
       </c>
       <c r="G69" s="28">
-        <v>4447.1</v>
+        <v>4268.85</v>
       </c>
       <c r="H69" s="29">
-        <v>0.0756</v>
+        <v>0.0726</v>
       </c>
       <c r="I69" s="29">
-        <v>0.0038</v>
+        <v>0.0037</v>
       </c>
       <c r="J69" s="29">
         <v>0.0054</v>
@@ -23576,16 +23576,16 @@
         <v>31068.3</v>
       </c>
       <c r="E72" s="28">
-        <v>1362.2</v>
+        <v>1362.85</v>
       </c>
       <c r="F72" s="28">
-        <v>58574.6</v>
+        <v>58602.55</v>
       </c>
       <c r="G72" s="28">
-        <v>27506.3</v>
+        <v>27534.25</v>
       </c>
       <c r="H72" s="29">
-        <v>0.8853</v>
+        <v>0.8862</v>
       </c>
       <c r="I72" s="29">
         <v>0.0035</v>
@@ -23752,16 +23752,16 @@
         <v>52499.2</v>
       </c>
       <c r="E76" s="28">
-        <v>380.3</v>
+        <v>381.4</v>
       </c>
       <c r="F76" s="28">
-        <v>55143.5</v>
+        <v>55154.5</v>
       </c>
       <c r="G76" s="28">
-        <v>2644.3</v>
+        <v>2655.3</v>
       </c>
       <c r="H76" s="29">
-        <v>0.0504</v>
+        <v>0.0506</v>
       </c>
       <c r="I76" s="29">
         <v>0.0033</v>
@@ -23972,16 +23972,16 @@
         <v>46569.23</v>
       </c>
       <c r="E81" s="28">
-        <v>224.8</v>
+        <v>225.35</v>
       </c>
       <c r="F81" s="28">
-        <v>48404.1</v>
+        <v>48409.05</v>
       </c>
       <c r="G81" s="28">
-        <v>1834.87</v>
+        <v>1839.82</v>
       </c>
       <c r="H81" s="29">
-        <v>0.0394</v>
+        <v>0.0395</v>
       </c>
       <c r="I81" s="29">
         <v>0.0029</v>
@@ -24060,16 +24060,16 @@
         <v>49689.7</v>
       </c>
       <c r="E83" s="28">
-        <v>850.9</v>
+        <v>851.45</v>
       </c>
       <c r="F83" s="28">
-        <v>46799.5</v>
+        <v>46829.75</v>
       </c>
       <c r="G83" s="28">
-        <v>-2890.2</v>
+        <v>-2859.95</v>
       </c>
       <c r="H83" s="29">
-        <v>-0.0582</v>
+        <v>-0.0576</v>
       </c>
       <c r="I83" s="29">
         <v>0.0028</v>
@@ -24456,16 +24456,16 @@
         <v>29686.25</v>
       </c>
       <c r="E92" s="28">
-        <v>796.0</v>
+        <v>800.8</v>
       </c>
       <c r="F92" s="28">
-        <v>35820.0</v>
+        <v>36036.0</v>
       </c>
       <c r="G92" s="28">
-        <v>6133.75</v>
+        <v>6349.75</v>
       </c>
       <c r="H92" s="29">
-        <v>0.2066</v>
+        <v>0.2139</v>
       </c>
       <c r="I92" s="29">
         <v>0.0021</v>
@@ -24547,13 +24547,13 @@
         <v>113.45</v>
       </c>
       <c r="F94" s="28">
-        <v>34824.3</v>
+        <v>34829.15</v>
       </c>
       <c r="G94" s="28">
-        <v>4987.06</v>
+        <v>4991.91</v>
       </c>
       <c r="H94" s="29">
-        <v>0.1671</v>
+        <v>0.1673</v>
       </c>
       <c r="I94" s="29">
         <v>0.0021</v>
@@ -24588,16 +24588,16 @@
         <v>33392.27</v>
       </c>
       <c r="E95" s="28">
-        <v>133.45</v>
+        <v>133.82</v>
       </c>
       <c r="F95" s="28">
-        <v>33229.05</v>
+        <v>33321.18</v>
       </c>
       <c r="G95" s="28">
-        <v>-163.22</v>
+        <v>-71.09</v>
       </c>
       <c r="H95" s="29">
-        <v>-0.0049</v>
+        <v>-0.0021</v>
       </c>
       <c r="I95" s="29">
         <v>0.002</v>
@@ -24723,13 +24723,13 @@
         <v>947.05</v>
       </c>
       <c r="F98" s="28">
-        <v>31222.9</v>
+        <v>31252.65</v>
       </c>
       <c r="G98" s="28">
-        <v>-4147.35</v>
+        <v>-4117.6</v>
       </c>
       <c r="H98" s="29">
-        <v>-0.1173</v>
+        <v>-0.1164</v>
       </c>
       <c r="I98" s="29">
         <v>0.0019</v>
@@ -24764,16 +24764,16 @@
         <v>12454.04</v>
       </c>
       <c r="E99" s="28">
-        <v>104.0</v>
+        <v>103.9</v>
       </c>
       <c r="F99" s="28">
-        <v>30992.0</v>
+        <v>30962.2</v>
       </c>
       <c r="G99" s="28">
-        <v>18537.96</v>
+        <v>18508.16</v>
       </c>
       <c r="H99" s="29">
-        <v>1.4885</v>
+        <v>1.4861</v>
       </c>
       <c r="I99" s="29">
         <v>0.0018</v>
@@ -24896,16 +24896,16 @@
         <v>25557.45</v>
       </c>
       <c r="E102" s="28">
-        <v>424.3</v>
+        <v>424.65</v>
       </c>
       <c r="F102" s="28">
-        <v>28003.8</v>
+        <v>28026.9</v>
       </c>
       <c r="G102" s="28">
-        <v>2446.35</v>
+        <v>2469.45</v>
       </c>
       <c r="H102" s="29">
-        <v>0.0957</v>
+        <v>0.0966</v>
       </c>
       <c r="I102" s="29">
         <v>0.0017</v>
@@ -25031,10 +25031,10 @@
         <v>527.0</v>
       </c>
       <c r="F105" s="28">
-        <v>26876.5</v>
+        <v>26877.0</v>
       </c>
       <c r="G105" s="28">
-        <v>1653.9</v>
+        <v>1654.4</v>
       </c>
       <c r="H105" s="29">
         <v>0.0656</v>
@@ -25072,16 +25072,16 @@
         <v>24907.3</v>
       </c>
       <c r="E106" s="28">
-        <v>620.5</v>
+        <v>620.75</v>
       </c>
       <c r="F106" s="28">
-        <v>26681.5</v>
+        <v>26692.25</v>
       </c>
       <c r="G106" s="28">
-        <v>1774.2</v>
+        <v>1784.95</v>
       </c>
       <c r="H106" s="29">
-        <v>0.0712</v>
+        <v>0.0717</v>
       </c>
       <c r="I106" s="29">
         <v>0.0016</v>
@@ -25116,13 +25116,13 @@
         <v>34032.35</v>
       </c>
       <c r="E107" s="28">
-        <v>437.9</v>
+        <v>437.45</v>
       </c>
       <c r="F107" s="28">
-        <v>25810.0</v>
+        <v>25809.55</v>
       </c>
       <c r="G107" s="28">
-        <v>-8222.35</v>
+        <v>-8222.8</v>
       </c>
       <c r="H107" s="29">
         <v>-0.2416</v>
@@ -25192,28 +25192,28 @@
     </row>
     <row r="109">
       <c r="A109" s="1" t="s">
-        <v>75</v>
+        <v>149</v>
       </c>
       <c r="B109" s="27">
-        <v>9.0</v>
+        <v>5.0</v>
       </c>
       <c r="C109" s="28">
-        <v>1395.0</v>
+        <v>2134.6</v>
       </c>
       <c r="D109" s="28">
-        <v>12555.0</v>
+        <v>10673.0</v>
       </c>
       <c r="E109" s="28">
-        <v>2574.0</v>
+        <v>4621.2</v>
       </c>
       <c r="F109" s="28">
-        <v>23166.0</v>
+        <v>23106.0</v>
       </c>
       <c r="G109" s="28">
-        <v>10611.0</v>
+        <v>12433.0</v>
       </c>
       <c r="H109" s="29">
-        <v>0.8452</v>
+        <v>1.1649</v>
       </c>
       <c r="I109" s="29">
         <v>0.0014</v>
@@ -25222,7 +25222,7 @@
         <v>0.002</v>
       </c>
       <c r="K109" s="1" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="L109" s="1" t="s">
         <v>16</v>
@@ -25236,37 +25236,37 @@
     </row>
     <row r="110">
       <c r="A110" s="1" t="s">
-        <v>149</v>
+        <v>75</v>
       </c>
       <c r="B110" s="27">
-        <v>5.0</v>
+        <v>9.0</v>
       </c>
       <c r="C110" s="28">
-        <v>2134.6</v>
+        <v>1395.0</v>
       </c>
       <c r="D110" s="28">
-        <v>10673.0</v>
+        <v>12555.0</v>
       </c>
       <c r="E110" s="28">
-        <v>4621.2</v>
+        <v>2537.0</v>
       </c>
       <c r="F110" s="28">
-        <v>23106.0</v>
+        <v>22833.0</v>
       </c>
       <c r="G110" s="28">
-        <v>12433.0</v>
+        <v>10278.0</v>
       </c>
       <c r="H110" s="29">
-        <v>1.1649</v>
+        <v>0.8186</v>
       </c>
       <c r="I110" s="29">
         <v>0.0014</v>
       </c>
       <c r="J110" s="29">
-        <v>0.002</v>
+        <v>0.0019</v>
       </c>
       <c r="K110" s="1" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="L110" s="1" t="s">
         <v>16</v>
@@ -25820,16 +25820,16 @@
         <v>19914.4</v>
       </c>
       <c r="E123" s="28">
-        <v>169.5</v>
+        <v>169.22</v>
       </c>
       <c r="F123" s="28">
-        <v>18645.0</v>
+        <v>18614.2</v>
       </c>
       <c r="G123" s="28">
-        <v>-1269.4</v>
+        <v>-1300.2</v>
       </c>
       <c r="H123" s="29">
-        <v>-0.0637</v>
+        <v>-0.0653</v>
       </c>
       <c r="I123" s="29">
         <v>0.0011</v>
@@ -25952,16 +25952,16 @@
         <v>14635.0</v>
       </c>
       <c r="E126" s="28">
-        <v>309.45</v>
+        <v>309.55</v>
       </c>
       <c r="F126" s="28">
-        <v>15472.5</v>
+        <v>15477.5</v>
       </c>
       <c r="G126" s="28">
-        <v>837.5</v>
+        <v>842.5</v>
       </c>
       <c r="H126" s="29">
-        <v>0.0572</v>
+        <v>0.0576</v>
       </c>
       <c r="I126" s="29">
         <v>9.0E-4</v>
@@ -26084,16 +26084,16 @@
         <v>9990.4</v>
       </c>
       <c r="E129" s="28">
-        <v>770.6</v>
+        <v>771.45</v>
       </c>
       <c r="F129" s="28">
-        <v>10788.4</v>
+        <v>10800.3</v>
       </c>
       <c r="G129" s="28">
-        <v>798.0</v>
+        <v>809.9</v>
       </c>
       <c r="H129" s="29">
-        <v>0.0799</v>
+        <v>0.0811</v>
       </c>
       <c r="I129" s="29">
         <v>6.0E-4</v>
@@ -26348,16 +26348,16 @@
         <v>3464.5</v>
       </c>
       <c r="E135" s="28">
-        <v>1892.0</v>
+        <v>1892.45</v>
       </c>
       <c r="F135" s="28">
-        <v>5676.0</v>
+        <v>5677.35</v>
       </c>
       <c r="G135" s="28">
-        <v>2211.5</v>
+        <v>2212.85</v>
       </c>
       <c r="H135" s="29">
-        <v>0.6383</v>
+        <v>0.6387</v>
       </c>
       <c r="I135" s="29">
         <v>3.0E-4</v>
@@ -26392,16 +26392,16 @@
         <v>4377.95</v>
       </c>
       <c r="E136" s="28">
-        <v>90.0</v>
+        <v>90.38</v>
       </c>
       <c r="F136" s="28">
-        <v>3510.0</v>
+        <v>3524.82</v>
       </c>
       <c r="G136" s="28">
-        <v>-867.95</v>
+        <v>-853.13</v>
       </c>
       <c r="H136" s="29">
-        <v>-0.1983</v>
+        <v>-0.1949</v>
       </c>
       <c r="I136" s="29">
         <v>2.0E-4</v>
@@ -26436,16 +26436,16 @@
         <v>885.9</v>
       </c>
       <c r="E137" s="28">
-        <v>314.5</v>
+        <v>314.9</v>
       </c>
       <c r="F137" s="28">
-        <v>3459.5</v>
+        <v>3463.9</v>
       </c>
       <c r="G137" s="28">
-        <v>2573.6</v>
+        <v>2578.0</v>
       </c>
       <c r="H137" s="29">
-        <v>2.9051</v>
+        <v>2.91</v>
       </c>
       <c r="I137" s="29">
         <v>2.0E-4</v>
@@ -26480,16 +26480,16 @@
         <v>415.9</v>
       </c>
       <c r="E138" s="28">
-        <v>1915.5</v>
+        <v>1915.7</v>
       </c>
       <c r="F138" s="28">
-        <v>1915.5</v>
+        <v>1915.7</v>
       </c>
       <c r="G138" s="28">
-        <v>1499.6</v>
+        <v>1499.8</v>
       </c>
       <c r="H138" s="29">
-        <v>3.6057</v>
+        <v>3.6062</v>
       </c>
       <c r="I138" s="29">
         <v>1.0E-4</v>
@@ -26524,16 +26524,16 @@
         <v>588.9</v>
       </c>
       <c r="E139" s="28">
-        <v>787.45</v>
+        <v>784.1</v>
       </c>
       <c r="F139" s="28">
-        <v>787.45</v>
+        <v>784.1</v>
       </c>
       <c r="G139" s="28">
-        <v>198.55</v>
+        <v>195.2</v>
       </c>
       <c r="H139" s="29">
-        <v>0.3372</v>
+        <v>0.3315</v>
       </c>
       <c r="I139" s="29">
         <v>0.0</v>
@@ -26568,16 +26568,16 @@
         <v>262.0</v>
       </c>
       <c r="E140" s="28">
-        <v>726.85</v>
+        <v>727.3</v>
       </c>
       <c r="F140" s="28">
-        <v>726.85</v>
+        <v>727.3</v>
       </c>
       <c r="G140" s="28">
-        <v>464.85</v>
+        <v>465.3</v>
       </c>
       <c r="H140" s="29">
-        <v>1.7742</v>
+        <v>1.776</v>
       </c>
       <c r="I140" s="29">
         <v>0.0</v>
@@ -26656,16 +26656,16 @@
         <v>53.6</v>
       </c>
       <c r="E142" s="28">
-        <v>514.3</v>
+        <v>514.55</v>
       </c>
       <c r="F142" s="28">
-        <v>514.3</v>
+        <v>514.55</v>
       </c>
       <c r="G142" s="28">
-        <v>460.7</v>
+        <v>460.95</v>
       </c>
       <c r="H142" s="29">
-        <v>8.5951</v>
+        <v>8.5998</v>
       </c>
       <c r="I142" s="29">
         <v>0.0</v>
@@ -26700,16 +26700,16 @@
         <v>222.45</v>
       </c>
       <c r="E143" s="28">
-        <v>385.8</v>
+        <v>386.55</v>
       </c>
       <c r="F143" s="28">
-        <v>385.8</v>
+        <v>386.55</v>
       </c>
       <c r="G143" s="28">
-        <v>163.35</v>
+        <v>164.1</v>
       </c>
       <c r="H143" s="29">
-        <v>0.7343</v>
+        <v>0.7377</v>
       </c>
       <c r="I143" s="29">
         <v>0.0</v>
@@ -26744,16 +26744,16 @@
         <v>394.05</v>
       </c>
       <c r="E144" s="28">
-        <v>334.7</v>
+        <v>334.4</v>
       </c>
       <c r="F144" s="28">
-        <v>334.7</v>
+        <v>334.4</v>
       </c>
       <c r="G144" s="28">
-        <v>-59.35</v>
+        <v>-59.65</v>
       </c>
       <c r="H144" s="29">
-        <v>-0.1506</v>
+        <v>-0.1514</v>
       </c>
       <c r="I144" s="29">
         <v>0.0</v>
@@ -26832,16 +26832,16 @@
         <v>165.85</v>
       </c>
       <c r="E146" s="28">
-        <v>289.4</v>
+        <v>289.85</v>
       </c>
       <c r="F146" s="28">
-        <v>289.4</v>
+        <v>289.85</v>
       </c>
       <c r="G146" s="28">
-        <v>123.55</v>
+        <v>124.0</v>
       </c>
       <c r="H146" s="29">
-        <v>0.745</v>
+        <v>0.7477</v>
       </c>
       <c r="I146" s="29">
         <v>0.0</v>
@@ -26964,16 +26964,16 @@
         <v>25.25</v>
       </c>
       <c r="E149" s="28">
-        <v>138.15</v>
+        <v>138.27</v>
       </c>
       <c r="F149" s="28">
-        <v>138.15</v>
+        <v>138.27</v>
       </c>
       <c r="G149" s="28">
-        <v>112.9</v>
+        <v>113.02</v>
       </c>
       <c r="H149" s="29">
-        <v>4.4713</v>
+        <v>4.476</v>
       </c>
       <c r="I149" s="29">
         <v>0.0</v>
@@ -27052,16 +27052,16 @@
         <v>51.86</v>
       </c>
       <c r="E151" s="28">
-        <v>96.59</v>
+        <v>96.9</v>
       </c>
       <c r="F151" s="28">
-        <v>96.59</v>
+        <v>96.9</v>
       </c>
       <c r="G151" s="28">
-        <v>44.73</v>
+        <v>45.04</v>
       </c>
       <c r="H151" s="29">
-        <v>0.8624</v>
+        <v>0.8684</v>
       </c>
       <c r="I151" s="29">
         <v>0.0</v>

</xml_diff>

<commit_message>
chore: refresh prices 2026-07-13 07:45 UTC
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3915" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3907" uniqueCount="231">
   <si>
     <t>Account Name</t>
   </si>
@@ -719,7 +719,7 @@
     <numFmt numFmtId="165" formatCode="[Green]#,##,##0;[Red]-#,##,##0"/>
     <numFmt numFmtId="166" formatCode="[Green]0%;[Red]-0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -762,6 +762,16 @@
       <sz val="11.0"/>
       <color rgb="FFF35631"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color rgb="FF1F3864"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
@@ -848,7 +858,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -948,10 +958,13 @@
     <xf borderId="0" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -15355,7 +15368,7 @@
         <v>17</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
     </row>
     <row r="76">
@@ -15932,8 +15945,8 @@
       <c r="D109" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="E109" s="10" t="s">
-        <v>17</v>
+      <c r="E109" s="33" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="110">
@@ -16766,11 +16779,11 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="33" t="s">
+      <c r="A159" s="34" t="s">
         <v>21</v>
       </c>
       <c r="B159" s="10" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C159" s="10" t="s">
         <v>16</v>
@@ -16781,16 +16794,13 @@
       <c r="E159" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F159" s="33" t="s">
-        <v>199</v>
-      </c>
     </row>
     <row r="160">
-      <c r="A160" s="33" t="s">
+      <c r="A160" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="B160" s="33" t="s">
-        <v>22</v>
+      <c r="B160" s="34" t="s">
+        <v>25</v>
       </c>
       <c r="C160" s="10" t="s">
         <v>16</v>
@@ -16798,19 +16808,16 @@
       <c r="D160" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="E160" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F160" s="33" t="s">
-        <v>199</v>
+      <c r="E160" s="33" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="33" t="s">
+      <c r="A161" s="34" t="s">
         <v>128</v>
       </c>
-      <c r="B161" s="33" t="s">
-        <v>22</v>
+      <c r="B161" s="34" t="s">
+        <v>25</v>
       </c>
       <c r="C161" s="10" t="s">
         <v>16</v>
@@ -16821,18 +16828,15 @@
       <c r="E161" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F161" s="33" t="s">
-        <v>199</v>
-      </c>
     </row>
     <row r="162">
-      <c r="A162" s="33" t="s">
+      <c r="A162" s="34" t="s">
         <v>141</v>
       </c>
-      <c r="B162" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C162" s="33" t="s">
+      <c r="B162" s="33" t="s">
+        <v>25</v>
+      </c>
+      <c r="C162" s="34" t="s">
         <v>16</v>
       </c>
       <c r="D162" s="10" t="s">
@@ -16841,18 +16845,15 @@
       <c r="E162" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F162" s="33" t="s">
-        <v>199</v>
-      </c>
     </row>
     <row r="163">
-      <c r="A163" s="33" t="s">
+      <c r="A163" s="34" t="s">
         <v>158</v>
       </c>
-      <c r="B163" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C163" s="33" t="s">
+      <c r="B163" s="33" t="s">
+        <v>25</v>
+      </c>
+      <c r="C163" s="34" t="s">
         <v>16</v>
       </c>
       <c r="D163" s="10" t="s">
@@ -16861,18 +16862,15 @@
       <c r="E163" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F163" s="33" t="s">
-        <v>199</v>
-      </c>
     </row>
     <row r="164">
-      <c r="A164" s="33" t="s">
+      <c r="A164" s="34" t="s">
         <v>194</v>
       </c>
-      <c r="B164" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C164" s="33" t="s">
+      <c r="B164" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="C164" s="34" t="s">
         <v>50</v>
       </c>
       <c r="D164" s="10" t="s">
@@ -16881,48 +16879,39 @@
       <c r="E164" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F164" s="33" t="s">
-        <v>199</v>
-      </c>
     </row>
     <row r="165">
-      <c r="A165" s="33" t="s">
+      <c r="A165" s="34" t="s">
         <v>196</v>
       </c>
       <c r="B165" s="33" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C165" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D165" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="E165" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="F165" s="33" t="s">
-        <v>199</v>
+      <c r="D165" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="E165" s="34" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="33" t="s">
+      <c r="A166" s="34" t="s">
         <v>195</v>
       </c>
       <c r="B166" s="33" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C166" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D166" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="E166" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="F166" s="33" t="s">
-        <v>199</v>
+      <c r="D166" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="E166" s="34" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -18065,28 +18054,28 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="34" t="s">
+      <c r="E1" s="35" t="s">
         <v>227</v>
       </c>
-      <c r="F1" s="34" t="s">
+      <c r="F1" s="35" t="s">
         <v>228</v>
       </c>
-      <c r="G1" s="34" t="s">
+      <c r="G1" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="34" t="s">
+      <c r="H1" s="35" t="s">
         <v>12</v>
       </c>
     </row>
@@ -20902,8 +20891,8 @@
       <c r="A110" s="4"/>
       <c r="B110" s="29"/>
       <c r="C110" s="29"/>
-      <c r="D110" s="35"/>
-      <c r="E110" s="36"/>
+      <c r="D110" s="36"/>
+      <c r="E110" s="37"/>
       <c r="F110" s="30"/>
       <c r="G110" s="4"/>
       <c r="H110" s="4"/>
@@ -20941,46 +20930,46 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="37" t="s">
+      <c r="B1" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="37" t="s">
+      <c r="C1" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="37" t="s">
+      <c r="D1" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="37" t="s">
+      <c r="E1" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="37" t="s">
+      <c r="F1" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="37" t="s">
+      <c r="G1" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="37" t="s">
+      <c r="H1" s="38" t="s">
         <v>227</v>
       </c>
-      <c r="I1" s="37" t="s">
+      <c r="I1" s="38" t="s">
         <v>228</v>
       </c>
-      <c r="J1" s="37" t="s">
+      <c r="J1" s="38" t="s">
         <v>229</v>
       </c>
-      <c r="K1" s="37" t="s">
+      <c r="K1" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="37" t="s">
+      <c r="L1" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="37" t="s">
+      <c r="M1" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="37" t="s">
+      <c r="N1" s="38" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>